<commit_message>
Update Singlish input types and evidence in Excel file
</commit_message>
<xml_diff>
--- a/IT23809642 - Test cases.xlsx
+++ b/IT23809642 - Test cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hashi\Downloads\IT23809642\test_automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B13730FD-4B94-4402-9D1C-C021C6A23B68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{333D265E-4A3E-4242-A57E-1E6635C964F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1182,7 +1182,7 @@
     <t>Rationale: Words like “purudu”, “ath ara” are romanized Sinhala</t>
   </si>
   <si>
-    <t>Evidence: Informal/casual structure used</t>
+    <t>Evidence: Informal/casual structure used.</t>
   </si>
 </sst>
 </file>
@@ -1324,23 +1324,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1363,6 +1346,23 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1655,7 +1655,7 @@
     <col min="5" max="5" width="31.88671875" style="1" customWidth="1"/>
     <col min="6" max="6" width="31.109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="8.88671875" style="1" customWidth="1"/>
-    <col min="8" max="9" width="38.109375" style="14" customWidth="1"/>
+    <col min="8" max="9" width="38.109375" style="7" customWidth="1"/>
     <col min="10" max="15" width="8.88671875" style="1" customWidth="1"/>
     <col min="16" max="16384" width="8.88671875" style="1"/>
   </cols>
@@ -1688,22 +1688,22 @@
       </c>
     </row>
     <row r="3" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="E3" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H3" s="5" t="s">
@@ -1714,12 +1714,12 @@
       </c>
     </row>
     <row r="4" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
       <c r="H4" s="5" t="s">
         <v>211</v>
       </c>
@@ -1728,12 +1728,12 @@
       </c>
     </row>
     <row r="5" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
       <c r="H5" s="5" t="s">
         <v>212</v>
       </c>
@@ -1742,12 +1742,12 @@
       </c>
     </row>
     <row r="6" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
       <c r="H6" s="6" t="s">
         <v>213</v>
       </c>
@@ -1756,22 +1756,22 @@
       </c>
     </row>
     <row r="7" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="E7" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H7" s="5" t="s">
@@ -1782,12 +1782,12 @@
       </c>
     </row>
     <row r="8" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
       <c r="H8" s="5" t="s">
         <v>212</v>
       </c>
@@ -1796,32 +1796,32 @@
       </c>
     </row>
     <row r="9" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
       <c r="H9" s="6"/>
       <c r="I9" s="6"/>
     </row>
     <row r="10" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H10" s="5" t="s">
@@ -1832,12 +1832,12 @@
       </c>
     </row>
     <row r="11" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
       <c r="H11" s="4" t="s">
         <v>216</v>
       </c>
@@ -1846,12 +1846,12 @@
       </c>
     </row>
     <row r="12" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
       <c r="H12" s="5" t="s">
         <v>217</v>
       </c>
@@ -1860,32 +1860,32 @@
       </c>
     </row>
     <row r="13" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
     </row>
     <row r="14" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D14" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="E14" s="12" t="s">
+      <c r="E14" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="F14" s="12" t="s">
+      <c r="F14" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="G14" s="7" t="s">
+      <c r="G14" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H14" s="5" t="s">
@@ -1896,12 +1896,12 @@
       </c>
     </row>
     <row r="15" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
       <c r="H15" s="5" t="s">
         <v>218</v>
       </c>
@@ -1910,32 +1910,32 @@
       </c>
     </row>
     <row r="16" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
       <c r="H16" s="6"/>
       <c r="I16" s="6"/>
     </row>
     <row r="17" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D17" s="12" t="s">
+      <c r="D17" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="E17" s="12" t="s">
+      <c r="E17" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="F17" s="12" t="s">
+      <c r="F17" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="G17" s="7" t="s">
+      <c r="G17" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H17" s="5" t="s">
@@ -1946,12 +1946,12 @@
       </c>
     </row>
     <row r="18" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
       <c r="H18" s="5" t="s">
         <v>219</v>
       </c>
@@ -1960,12 +1960,12 @@
       </c>
     </row>
     <row r="19" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
       <c r="H19" s="5" t="s">
         <v>218</v>
       </c>
@@ -1974,32 +1974,32 @@
       </c>
     </row>
     <row r="20" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
       <c r="H20" s="6"/>
       <c r="I20" s="6"/>
     </row>
     <row r="21" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="D21" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="E21" s="12" t="s">
+      <c r="E21" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="F21" s="12" t="s">
+      <c r="F21" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="G21" s="7" t="s">
+      <c r="G21" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H21" s="5" t="s">
@@ -2010,12 +2010,12 @@
       </c>
     </row>
     <row r="22" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
+      <c r="B22" s="16"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="16"/>
       <c r="H22" s="5" t="s">
         <v>221</v>
       </c>
@@ -2024,12 +2024,12 @@
       </c>
     </row>
     <row r="23" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="16"/>
       <c r="H23" s="5" t="s">
         <v>218</v>
       </c>
@@ -2038,32 +2038,32 @@
       </c>
     </row>
     <row r="24" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
       <c r="H24" s="6"/>
       <c r="I24" s="6"/>
     </row>
     <row r="25" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="E25" s="12" t="s">
+      <c r="E25" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="F25" s="12" t="s">
+      <c r="F25" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="G25" s="7" t="s">
+      <c r="G25" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H25" s="5" t="s">
@@ -2074,12 +2074,12 @@
       </c>
     </row>
     <row r="26" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="16"/>
+      <c r="G26" s="16"/>
       <c r="H26" s="5" t="s">
         <v>219</v>
       </c>
@@ -2088,12 +2088,12 @@
       </c>
     </row>
     <row r="27" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="8"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="8"/>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
+      <c r="B27" s="16"/>
+      <c r="C27" s="16"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="16"/>
+      <c r="G27" s="16"/>
       <c r="H27" s="5" t="s">
         <v>218</v>
       </c>
@@ -2102,32 +2102,32 @@
       </c>
     </row>
     <row r="28" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="9"/>
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-      <c r="G28" s="9"/>
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="17"/>
       <c r="H28" s="6"/>
       <c r="I28" s="6"/>
     </row>
     <row r="29" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="11" t="s">
+      <c r="B29" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="C29" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D29" s="12" t="s">
+      <c r="D29" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="E29" s="12" t="s">
+      <c r="E29" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="F29" s="12" t="s">
+      <c r="F29" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="G29" s="7" t="s">
+      <c r="G29" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H29" s="5" t="s">
@@ -2138,12 +2138,12 @@
       </c>
     </row>
     <row r="30" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="8"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
-      <c r="F30" s="8"/>
-      <c r="G30" s="8"/>
+      <c r="B30" s="16"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="16"/>
       <c r="H30" s="5" t="s">
         <v>220</v>
       </c>
@@ -2152,13 +2152,13 @@
       </c>
     </row>
     <row r="31" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="8"/>
-      <c r="C31" s="8"/>
-      <c r="D31" s="8"/>
-      <c r="E31" s="8"/>
-      <c r="F31" s="8"/>
-      <c r="G31" s="8"/>
-      <c r="H31" s="14" t="s">
+      <c r="B31" s="16"/>
+      <c r="C31" s="16"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
+      <c r="G31" s="16"/>
+      <c r="H31" s="7" t="s">
         <v>218</v>
       </c>
       <c r="I31" s="5" t="s">
@@ -2166,32 +2166,32 @@
       </c>
     </row>
     <row r="32" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="9"/>
-      <c r="C32" s="9"/>
-      <c r="D32" s="9"/>
-      <c r="E32" s="9"/>
-      <c r="F32" s="9"/>
-      <c r="G32" s="9"/>
+      <c r="B32" s="17"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="17"/>
       <c r="H32" s="6"/>
       <c r="I32" s="6"/>
     </row>
     <row r="33" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="11" t="s">
+      <c r="B33" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="C33" s="7" t="s">
+      <c r="C33" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D33" s="12" t="s">
+      <c r="D33" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="E33" s="12" t="s">
+      <c r="E33" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="F33" s="12" t="s">
+      <c r="F33" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="G33" s="7" t="s">
+      <c r="G33" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H33" s="5" t="s">
@@ -2202,12 +2202,12 @@
       </c>
     </row>
     <row r="34" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="8"/>
-      <c r="C34" s="8"/>
-      <c r="D34" s="8"/>
-      <c r="E34" s="8"/>
-      <c r="F34" s="8"/>
-      <c r="G34" s="8"/>
+      <c r="B34" s="16"/>
+      <c r="C34" s="16"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
+      <c r="F34" s="16"/>
+      <c r="G34" s="16"/>
       <c r="H34" s="5" t="s">
         <v>212</v>
       </c>
@@ -2216,12 +2216,12 @@
       </c>
     </row>
     <row r="35" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="8"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
-      <c r="E35" s="8"/>
-      <c r="F35" s="8"/>
-      <c r="G35" s="8"/>
+      <c r="B35" s="16"/>
+      <c r="C35" s="16"/>
+      <c r="D35" s="16"/>
+      <c r="E35" s="16"/>
+      <c r="F35" s="16"/>
+      <c r="G35" s="16"/>
       <c r="H35" s="5" t="s">
         <v>218</v>
       </c>
@@ -2230,32 +2230,32 @@
       </c>
     </row>
     <row r="36" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B36" s="9"/>
-      <c r="C36" s="9"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-      <c r="G36" s="9"/>
+      <c r="B36" s="17"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="17"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="17"/>
       <c r="H36" s="6"/>
       <c r="I36" s="6"/>
     </row>
     <row r="37" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="11" t="s">
+      <c r="B37" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="C37" s="7" t="s">
+      <c r="C37" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="D37" s="10" t="s">
+      <c r="D37" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="E37" s="10" t="s">
+      <c r="E37" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="F37" s="12" t="s">
+      <c r="F37" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="G37" s="7" t="s">
+      <c r="G37" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H37" s="5" t="s">
@@ -2266,12 +2266,12 @@
       </c>
     </row>
     <row r="38" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="8"/>
-      <c r="C38" s="8"/>
-      <c r="D38" s="8"/>
-      <c r="E38" s="8"/>
-      <c r="F38" s="8"/>
-      <c r="G38" s="8"/>
+      <c r="B38" s="16"/>
+      <c r="C38" s="16"/>
+      <c r="D38" s="16"/>
+      <c r="E38" s="16"/>
+      <c r="F38" s="16"/>
+      <c r="G38" s="16"/>
       <c r="H38" s="5" t="s">
         <v>221</v>
       </c>
@@ -2280,12 +2280,12 @@
       </c>
     </row>
     <row r="39" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="8"/>
-      <c r="C39" s="8"/>
-      <c r="D39" s="8"/>
-      <c r="E39" s="8"/>
-      <c r="F39" s="8"/>
-      <c r="G39" s="8"/>
+      <c r="B39" s="16"/>
+      <c r="C39" s="16"/>
+      <c r="D39" s="16"/>
+      <c r="E39" s="16"/>
+      <c r="F39" s="16"/>
+      <c r="G39" s="16"/>
       <c r="H39" s="5" t="s">
         <v>212</v>
       </c>
@@ -2294,12 +2294,12 @@
       </c>
     </row>
     <row r="40" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B40" s="8"/>
-      <c r="C40" s="8"/>
-      <c r="D40" s="8"/>
-      <c r="E40" s="8"/>
-      <c r="F40" s="8"/>
-      <c r="G40" s="8"/>
+      <c r="B40" s="16"/>
+      <c r="C40" s="16"/>
+      <c r="D40" s="16"/>
+      <c r="E40" s="16"/>
+      <c r="F40" s="16"/>
+      <c r="G40" s="16"/>
       <c r="H40" s="5" t="s">
         <v>210</v>
       </c>
@@ -2308,12 +2308,12 @@
       </c>
     </row>
     <row r="41" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B41" s="9"/>
-      <c r="C41" s="9"/>
-      <c r="D41" s="9"/>
-      <c r="E41" s="9"/>
-      <c r="F41" s="9"/>
-      <c r="G41" s="9"/>
+      <c r="B41" s="17"/>
+      <c r="C41" s="17"/>
+      <c r="D41" s="17"/>
+      <c r="E41" s="17"/>
+      <c r="F41" s="17"/>
+      <c r="G41" s="17"/>
       <c r="H41" s="6" t="s">
         <v>218</v>
       </c>
@@ -2322,22 +2322,22 @@
       </c>
     </row>
     <row r="42" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="11" t="s">
+      <c r="B42" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="C42" s="7" t="s">
+      <c r="C42" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D42" s="10" t="s">
+      <c r="D42" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="E42" s="10" t="s">
+      <c r="E42" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="F42" s="12" t="s">
+      <c r="F42" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="G42" s="7" t="s">
+      <c r="G42" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H42" s="5" t="s">
@@ -2348,12 +2348,12 @@
       </c>
     </row>
     <row r="43" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B43" s="8"/>
-      <c r="C43" s="8"/>
-      <c r="D43" s="8"/>
-      <c r="E43" s="8"/>
-      <c r="F43" s="8"/>
-      <c r="G43" s="8"/>
+      <c r="B43" s="16"/>
+      <c r="C43" s="16"/>
+      <c r="D43" s="16"/>
+      <c r="E43" s="16"/>
+      <c r="F43" s="16"/>
+      <c r="G43" s="16"/>
       <c r="H43" s="5" t="s">
         <v>219</v>
       </c>
@@ -2362,12 +2362,12 @@
       </c>
     </row>
     <row r="44" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B44" s="8"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="8"/>
-      <c r="F44" s="8"/>
-      <c r="G44" s="8"/>
+      <c r="B44" s="16"/>
+      <c r="C44" s="16"/>
+      <c r="D44" s="16"/>
+      <c r="E44" s="16"/>
+      <c r="F44" s="16"/>
+      <c r="G44" s="16"/>
       <c r="H44" s="5" t="s">
         <v>212</v>
       </c>
@@ -2376,12 +2376,12 @@
       </c>
     </row>
     <row r="45" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B45" s="9"/>
-      <c r="C45" s="9"/>
-      <c r="D45" s="9"/>
-      <c r="E45" s="9"/>
-      <c r="F45" s="9"/>
-      <c r="G45" s="9"/>
+      <c r="B45" s="17"/>
+      <c r="C45" s="17"/>
+      <c r="D45" s="17"/>
+      <c r="E45" s="17"/>
+      <c r="F45" s="17"/>
+      <c r="G45" s="17"/>
       <c r="H45" s="6" t="s">
         <v>218</v>
       </c>
@@ -2390,22 +2390,22 @@
       </c>
     </row>
     <row r="46" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B46" s="11" t="s">
+      <c r="B46" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="C46" s="7" t="s">
+      <c r="C46" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D46" s="10" t="s">
+      <c r="D46" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="E46" s="10" t="s">
+      <c r="E46" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="F46" s="12" t="s">
+      <c r="F46" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="G46" s="7" t="s">
+      <c r="G46" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H46" s="5" t="s">
@@ -2416,12 +2416,12 @@
       </c>
     </row>
     <row r="47" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B47" s="8"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="8"/>
-      <c r="E47" s="8"/>
-      <c r="F47" s="8"/>
-      <c r="G47" s="8"/>
+      <c r="B47" s="16"/>
+      <c r="C47" s="16"/>
+      <c r="D47" s="16"/>
+      <c r="E47" s="16"/>
+      <c r="F47" s="16"/>
+      <c r="G47" s="16"/>
       <c r="H47" s="5" t="s">
         <v>212</v>
       </c>
@@ -2430,12 +2430,12 @@
       </c>
     </row>
     <row r="48" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B48" s="8"/>
-      <c r="C48" s="8"/>
-      <c r="D48" s="8"/>
-      <c r="E48" s="8"/>
-      <c r="F48" s="8"/>
-      <c r="G48" s="8"/>
+      <c r="B48" s="16"/>
+      <c r="C48" s="16"/>
+      <c r="D48" s="16"/>
+      <c r="E48" s="16"/>
+      <c r="F48" s="16"/>
+      <c r="G48" s="16"/>
       <c r="H48" s="5" t="s">
         <v>218</v>
       </c>
@@ -2444,32 +2444,32 @@
       </c>
     </row>
     <row r="49" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B49" s="9"/>
-      <c r="C49" s="9"/>
-      <c r="D49" s="9"/>
-      <c r="E49" s="9"/>
-      <c r="F49" s="9"/>
-      <c r="G49" s="9"/>
+      <c r="B49" s="17"/>
+      <c r="C49" s="17"/>
+      <c r="D49" s="17"/>
+      <c r="E49" s="17"/>
+      <c r="F49" s="17"/>
+      <c r="G49" s="17"/>
       <c r="H49" s="6"/>
       <c r="I49" s="6"/>
     </row>
     <row r="50" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B50" s="11" t="s">
+      <c r="B50" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="C50" s="7" t="s">
+      <c r="C50" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D50" s="10" t="s">
+      <c r="D50" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="E50" s="10" t="s">
+      <c r="E50" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="F50" s="12" t="s">
+      <c r="F50" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="G50" s="7" t="s">
+      <c r="G50" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H50" s="5" t="s">
@@ -2480,12 +2480,12 @@
       </c>
     </row>
     <row r="51" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B51" s="8"/>
-      <c r="C51" s="8"/>
-      <c r="D51" s="8"/>
-      <c r="E51" s="8"/>
-      <c r="F51" s="8"/>
-      <c r="G51" s="8"/>
+      <c r="B51" s="16"/>
+      <c r="C51" s="16"/>
+      <c r="D51" s="16"/>
+      <c r="E51" s="16"/>
+      <c r="F51" s="16"/>
+      <c r="G51" s="16"/>
       <c r="H51" s="5" t="s">
         <v>218</v>
       </c>
@@ -2494,12 +2494,12 @@
       </c>
     </row>
     <row r="52" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B52" s="8"/>
-      <c r="C52" s="8"/>
-      <c r="D52" s="8"/>
-      <c r="E52" s="8"/>
-      <c r="F52" s="8"/>
-      <c r="G52" s="8"/>
+      <c r="B52" s="16"/>
+      <c r="C52" s="16"/>
+      <c r="D52" s="16"/>
+      <c r="E52" s="16"/>
+      <c r="F52" s="16"/>
+      <c r="G52" s="16"/>
       <c r="H52" s="5" t="s">
         <v>212</v>
       </c>
@@ -2508,32 +2508,32 @@
       </c>
     </row>
     <row r="53" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B53" s="9"/>
-      <c r="C53" s="9"/>
-      <c r="D53" s="9"/>
-      <c r="E53" s="9"/>
-      <c r="F53" s="9"/>
-      <c r="G53" s="9"/>
+      <c r="B53" s="17"/>
+      <c r="C53" s="17"/>
+      <c r="D53" s="17"/>
+      <c r="E53" s="17"/>
+      <c r="F53" s="17"/>
+      <c r="G53" s="17"/>
       <c r="H53" s="6"/>
       <c r="I53" s="6"/>
     </row>
     <row r="54" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B54" s="11" t="s">
+      <c r="B54" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="C54" s="7" t="s">
+      <c r="C54" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D54" s="10" t="s">
+      <c r="D54" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="E54" s="10" t="s">
+      <c r="E54" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="F54" s="12" t="s">
+      <c r="F54" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="G54" s="7" t="s">
+      <c r="G54" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H54" s="5" t="s">
@@ -2544,12 +2544,12 @@
       </c>
     </row>
     <row r="55" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B55" s="8"/>
-      <c r="C55" s="8"/>
-      <c r="D55" s="8"/>
-      <c r="E55" s="8"/>
-      <c r="F55" s="8"/>
-      <c r="G55" s="8"/>
+      <c r="B55" s="16"/>
+      <c r="C55" s="16"/>
+      <c r="D55" s="16"/>
+      <c r="E55" s="16"/>
+      <c r="F55" s="16"/>
+      <c r="G55" s="16"/>
       <c r="H55" s="5" t="s">
         <v>218</v>
       </c>
@@ -2558,12 +2558,12 @@
       </c>
     </row>
     <row r="56" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B56" s="8"/>
-      <c r="C56" s="8"/>
-      <c r="D56" s="8"/>
-      <c r="E56" s="8"/>
-      <c r="F56" s="8"/>
-      <c r="G56" s="8"/>
+      <c r="B56" s="16"/>
+      <c r="C56" s="16"/>
+      <c r="D56" s="16"/>
+      <c r="E56" s="16"/>
+      <c r="F56" s="16"/>
+      <c r="G56" s="16"/>
       <c r="H56" s="5" t="s">
         <v>212</v>
       </c>
@@ -2572,32 +2572,32 @@
       </c>
     </row>
     <row r="57" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B57" s="9"/>
-      <c r="C57" s="9"/>
-      <c r="D57" s="9"/>
-      <c r="E57" s="9"/>
-      <c r="F57" s="9"/>
-      <c r="G57" s="9"/>
+      <c r="B57" s="17"/>
+      <c r="C57" s="17"/>
+      <c r="D57" s="17"/>
+      <c r="E57" s="17"/>
+      <c r="F57" s="17"/>
+      <c r="G57" s="17"/>
       <c r="H57" s="6"/>
       <c r="I57" s="6"/>
     </row>
     <row r="58" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B58" s="11" t="s">
+      <c r="B58" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="C58" s="7" t="s">
+      <c r="C58" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D58" s="10" t="s">
+      <c r="D58" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="E58" s="10" t="s">
+      <c r="E58" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="F58" s="12" t="s">
+      <c r="F58" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="G58" s="7" t="s">
+      <c r="G58" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H58" s="5" t="s">
@@ -2608,12 +2608,12 @@
       </c>
     </row>
     <row r="59" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B59" s="8"/>
-      <c r="C59" s="8"/>
-      <c r="D59" s="8"/>
-      <c r="E59" s="8"/>
-      <c r="F59" s="8"/>
-      <c r="G59" s="8"/>
+      <c r="B59" s="16"/>
+      <c r="C59" s="16"/>
+      <c r="D59" s="16"/>
+      <c r="E59" s="16"/>
+      <c r="F59" s="16"/>
+      <c r="G59" s="16"/>
       <c r="H59" s="5" t="s">
         <v>210</v>
       </c>
@@ -2622,12 +2622,12 @@
       </c>
     </row>
     <row r="60" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B60" s="8"/>
-      <c r="C60" s="8"/>
-      <c r="D60" s="8"/>
-      <c r="E60" s="8"/>
-      <c r="F60" s="8"/>
-      <c r="G60" s="8"/>
+      <c r="B60" s="16"/>
+      <c r="C60" s="16"/>
+      <c r="D60" s="16"/>
+      <c r="E60" s="16"/>
+      <c r="F60" s="16"/>
+      <c r="G60" s="16"/>
       <c r="H60" s="5" t="s">
         <v>219</v>
       </c>
@@ -2636,12 +2636,12 @@
       </c>
     </row>
     <row r="61" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B61" s="9"/>
-      <c r="C61" s="9"/>
-      <c r="D61" s="9"/>
-      <c r="E61" s="9"/>
-      <c r="F61" s="9"/>
-      <c r="G61" s="9"/>
+      <c r="B61" s="17"/>
+      <c r="C61" s="17"/>
+      <c r="D61" s="17"/>
+      <c r="E61" s="17"/>
+      <c r="F61" s="17"/>
+      <c r="G61" s="17"/>
       <c r="H61" s="6" t="s">
         <v>218</v>
       </c>
@@ -2650,22 +2650,22 @@
       </c>
     </row>
     <row r="62" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B62" s="11" t="s">
+      <c r="B62" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="C62" s="7" t="s">
+      <c r="C62" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D62" s="10" t="s">
+      <c r="D62" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="E62" s="10" t="s">
+      <c r="E62" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="F62" s="12" t="s">
+      <c r="F62" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="G62" s="7" t="s">
+      <c r="G62" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H62" s="5" t="s">
@@ -2676,12 +2676,12 @@
       </c>
     </row>
     <row r="63" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B63" s="8"/>
-      <c r="C63" s="8"/>
-      <c r="D63" s="8"/>
-      <c r="E63" s="8"/>
-      <c r="F63" s="8"/>
-      <c r="G63" s="8"/>
+      <c r="B63" s="16"/>
+      <c r="C63" s="16"/>
+      <c r="D63" s="16"/>
+      <c r="E63" s="16"/>
+      <c r="F63" s="16"/>
+      <c r="G63" s="16"/>
       <c r="H63" s="5" t="s">
         <v>219</v>
       </c>
@@ -2690,13 +2690,13 @@
       </c>
     </row>
     <row r="64" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B64" s="8"/>
-      <c r="C64" s="8"/>
-      <c r="D64" s="8"/>
-      <c r="E64" s="8"/>
-      <c r="F64" s="8"/>
-      <c r="G64" s="8"/>
-      <c r="H64" s="16" t="s">
+      <c r="B64" s="16"/>
+      <c r="C64" s="16"/>
+      <c r="D64" s="16"/>
+      <c r="E64" s="16"/>
+      <c r="F64" s="16"/>
+      <c r="G64" s="16"/>
+      <c r="H64" s="9" t="s">
         <v>225</v>
       </c>
       <c r="I64" s="5" t="s">
@@ -2704,12 +2704,12 @@
       </c>
     </row>
     <row r="65" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B65" s="9"/>
-      <c r="C65" s="9"/>
-      <c r="D65" s="9"/>
-      <c r="E65" s="9"/>
-      <c r="F65" s="9"/>
-      <c r="G65" s="9"/>
+      <c r="B65" s="17"/>
+      <c r="C65" s="17"/>
+      <c r="D65" s="17"/>
+      <c r="E65" s="17"/>
+      <c r="F65" s="17"/>
+      <c r="G65" s="17"/>
       <c r="H65" s="6" t="s">
         <v>218</v>
       </c>
@@ -2718,22 +2718,22 @@
       </c>
     </row>
     <row r="66" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B66" s="11" t="s">
+      <c r="B66" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="C66" s="7" t="s">
+      <c r="C66" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D66" s="10" t="s">
+      <c r="D66" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="E66" s="10" t="s">
+      <c r="E66" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="F66" s="12" t="s">
+      <c r="F66" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="G66" s="7" t="s">
+      <c r="G66" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H66" s="5" t="s">
@@ -2744,12 +2744,12 @@
       </c>
     </row>
     <row r="67" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B67" s="8"/>
-      <c r="C67" s="8"/>
-      <c r="D67" s="8"/>
-      <c r="E67" s="8"/>
-      <c r="F67" s="8"/>
-      <c r="G67" s="8"/>
+      <c r="B67" s="16"/>
+      <c r="C67" s="16"/>
+      <c r="D67" s="16"/>
+      <c r="E67" s="16"/>
+      <c r="F67" s="16"/>
+      <c r="G67" s="16"/>
       <c r="H67" s="5" t="s">
         <v>226</v>
       </c>
@@ -2758,12 +2758,12 @@
       </c>
     </row>
     <row r="68" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B68" s="8"/>
-      <c r="C68" s="8"/>
-      <c r="D68" s="8"/>
-      <c r="E68" s="8"/>
-      <c r="F68" s="8"/>
-      <c r="G68" s="8"/>
+      <c r="B68" s="16"/>
+      <c r="C68" s="16"/>
+      <c r="D68" s="16"/>
+      <c r="E68" s="16"/>
+      <c r="F68" s="16"/>
+      <c r="G68" s="16"/>
       <c r="H68" s="5" t="s">
         <v>223</v>
       </c>
@@ -2772,12 +2772,12 @@
       </c>
     </row>
     <row r="69" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B69" s="9"/>
-      <c r="C69" s="9"/>
-      <c r="D69" s="9"/>
-      <c r="E69" s="9"/>
-      <c r="F69" s="9"/>
-      <c r="G69" s="9"/>
+      <c r="B69" s="17"/>
+      <c r="C69" s="17"/>
+      <c r="D69" s="17"/>
+      <c r="E69" s="17"/>
+      <c r="F69" s="17"/>
+      <c r="G69" s="17"/>
       <c r="H69" s="6" t="s">
         <v>218</v>
       </c>
@@ -2786,22 +2786,22 @@
       </c>
     </row>
     <row r="70" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B70" s="11" t="s">
+      <c r="B70" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="C70" s="7" t="s">
+      <c r="C70" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D70" s="10" t="s">
+      <c r="D70" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="E70" s="10" t="s">
+      <c r="E70" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="F70" s="12" t="s">
+      <c r="F70" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="G70" s="7" t="s">
+      <c r="G70" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H70" s="5" t="s">
@@ -2812,12 +2812,12 @@
       </c>
     </row>
     <row r="71" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B71" s="8"/>
-      <c r="C71" s="8"/>
-      <c r="D71" s="8"/>
-      <c r="E71" s="8"/>
-      <c r="F71" s="8"/>
-      <c r="G71" s="8"/>
+      <c r="B71" s="16"/>
+      <c r="C71" s="16"/>
+      <c r="D71" s="16"/>
+      <c r="E71" s="16"/>
+      <c r="F71" s="16"/>
+      <c r="G71" s="16"/>
       <c r="H71" s="5" t="s">
         <v>227</v>
       </c>
@@ -2826,12 +2826,12 @@
       </c>
     </row>
     <row r="72" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B72" s="8"/>
-      <c r="C72" s="8"/>
-      <c r="D72" s="8"/>
-      <c r="E72" s="8"/>
-      <c r="F72" s="8"/>
-      <c r="G72" s="8"/>
+      <c r="B72" s="16"/>
+      <c r="C72" s="16"/>
+      <c r="D72" s="16"/>
+      <c r="E72" s="16"/>
+      <c r="F72" s="16"/>
+      <c r="G72" s="16"/>
       <c r="H72" s="5" t="s">
         <v>216</v>
       </c>
@@ -2840,12 +2840,12 @@
       </c>
     </row>
     <row r="73" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B73" s="9"/>
-      <c r="C73" s="9"/>
-      <c r="D73" s="9"/>
-      <c r="E73" s="9"/>
-      <c r="F73" s="9"/>
-      <c r="G73" s="9"/>
+      <c r="B73" s="17"/>
+      <c r="C73" s="17"/>
+      <c r="D73" s="17"/>
+      <c r="E73" s="17"/>
+      <c r="F73" s="17"/>
+      <c r="G73" s="17"/>
       <c r="H73" s="6" t="s">
         <v>218</v>
       </c>
@@ -2854,22 +2854,22 @@
       </c>
     </row>
     <row r="74" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B74" s="11" t="s">
+      <c r="B74" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="C74" s="7" t="s">
+      <c r="C74" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D74" s="10" t="s">
+      <c r="D74" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="E74" s="10" t="s">
+      <c r="E74" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="F74" s="12" t="s">
+      <c r="F74" s="19" t="s">
         <v>84</v>
       </c>
-      <c r="G74" s="7" t="s">
+      <c r="G74" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H74" s="5" t="s">
@@ -2880,13 +2880,13 @@
       </c>
     </row>
     <row r="75" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B75" s="8"/>
-      <c r="C75" s="8"/>
-      <c r="D75" s="8"/>
-      <c r="E75" s="8"/>
-      <c r="F75" s="8"/>
-      <c r="G75" s="8"/>
-      <c r="H75" s="14" t="s">
+      <c r="B75" s="16"/>
+      <c r="C75" s="16"/>
+      <c r="D75" s="16"/>
+      <c r="E75" s="16"/>
+      <c r="F75" s="16"/>
+      <c r="G75" s="16"/>
+      <c r="H75" s="7" t="s">
         <v>216</v>
       </c>
       <c r="I75" s="5" t="s">
@@ -2894,12 +2894,12 @@
       </c>
     </row>
     <row r="76" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B76" s="8"/>
-      <c r="C76" s="8"/>
-      <c r="D76" s="8"/>
-      <c r="E76" s="8"/>
-      <c r="F76" s="8"/>
-      <c r="G76" s="8"/>
+      <c r="B76" s="16"/>
+      <c r="C76" s="16"/>
+      <c r="D76" s="16"/>
+      <c r="E76" s="16"/>
+      <c r="F76" s="16"/>
+      <c r="G76" s="16"/>
       <c r="H76" s="5" t="s">
         <v>217</v>
       </c>
@@ -2908,12 +2908,12 @@
       </c>
     </row>
     <row r="77" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B77" s="9"/>
-      <c r="C77" s="9"/>
-      <c r="D77" s="9"/>
-      <c r="E77" s="9"/>
-      <c r="F77" s="9"/>
-      <c r="G77" s="9"/>
+      <c r="B77" s="17"/>
+      <c r="C77" s="17"/>
+      <c r="D77" s="17"/>
+      <c r="E77" s="17"/>
+      <c r="F77" s="17"/>
+      <c r="G77" s="17"/>
       <c r="H77" s="6" t="s">
         <v>218</v>
       </c>
@@ -2922,22 +2922,22 @@
       </c>
     </row>
     <row r="78" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B78" s="11" t="s">
+      <c r="B78" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="C78" s="7" t="s">
+      <c r="C78" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D78" s="10" t="s">
+      <c r="D78" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="E78" s="10" t="s">
+      <c r="E78" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="F78" s="12" t="s">
+      <c r="F78" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="G78" s="7" t="s">
+      <c r="G78" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H78" s="5" t="s">
@@ -2948,12 +2948,12 @@
       </c>
     </row>
     <row r="79" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B79" s="8"/>
-      <c r="C79" s="8"/>
-      <c r="D79" s="8"/>
-      <c r="E79" s="8"/>
-      <c r="F79" s="8"/>
-      <c r="G79" s="8"/>
+      <c r="B79" s="16"/>
+      <c r="C79" s="16"/>
+      <c r="D79" s="16"/>
+      <c r="E79" s="16"/>
+      <c r="F79" s="16"/>
+      <c r="G79" s="16"/>
       <c r="H79" s="5" t="s">
         <v>219</v>
       </c>
@@ -2962,12 +2962,12 @@
       </c>
     </row>
     <row r="80" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B80" s="8"/>
-      <c r="C80" s="8"/>
-      <c r="D80" s="8"/>
-      <c r="E80" s="8"/>
-      <c r="F80" s="8"/>
-      <c r="G80" s="8"/>
+      <c r="B80" s="16"/>
+      <c r="C80" s="16"/>
+      <c r="D80" s="16"/>
+      <c r="E80" s="16"/>
+      <c r="F80" s="16"/>
+      <c r="G80" s="16"/>
       <c r="H80" s="5" t="s">
         <v>228</v>
       </c>
@@ -2976,12 +2976,12 @@
       </c>
     </row>
     <row r="81" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B81" s="9"/>
-      <c r="C81" s="9"/>
-      <c r="D81" s="9"/>
-      <c r="E81" s="9"/>
-      <c r="F81" s="9"/>
-      <c r="G81" s="9"/>
+      <c r="B81" s="17"/>
+      <c r="C81" s="17"/>
+      <c r="D81" s="17"/>
+      <c r="E81" s="17"/>
+      <c r="F81" s="17"/>
+      <c r="G81" s="17"/>
       <c r="H81" s="6" t="s">
         <v>229</v>
       </c>
@@ -2990,22 +2990,22 @@
       </c>
     </row>
     <row r="82" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B82" s="11" t="s">
+      <c r="B82" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="C82" s="7" t="s">
+      <c r="C82" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D82" s="10" t="s">
+      <c r="D82" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="E82" s="10" t="s">
+      <c r="E82" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="F82" s="12" t="s">
+      <c r="F82" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="G82" s="7" t="s">
+      <c r="G82" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H82" s="5" t="s">
@@ -3016,13 +3016,13 @@
       </c>
     </row>
     <row r="83" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B83" s="8"/>
-      <c r="C83" s="8"/>
-      <c r="D83" s="8"/>
-      <c r="E83" s="8"/>
-      <c r="F83" s="8"/>
-      <c r="G83" s="8"/>
-      <c r="H83" s="14" t="s">
+      <c r="B83" s="16"/>
+      <c r="C83" s="16"/>
+      <c r="D83" s="16"/>
+      <c r="E83" s="16"/>
+      <c r="F83" s="16"/>
+      <c r="G83" s="16"/>
+      <c r="H83" s="7" t="s">
         <v>219</v>
       </c>
       <c r="I83" s="5" t="s">
@@ -3030,13 +3030,13 @@
       </c>
     </row>
     <row r="84" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B84" s="8"/>
-      <c r="C84" s="8"/>
-      <c r="D84" s="8"/>
-      <c r="E84" s="8"/>
-      <c r="F84" s="8"/>
-      <c r="G84" s="8"/>
-      <c r="H84" s="15" t="s">
+      <c r="B84" s="16"/>
+      <c r="C84" s="16"/>
+      <c r="D84" s="16"/>
+      <c r="E84" s="16"/>
+      <c r="F84" s="16"/>
+      <c r="G84" s="16"/>
+      <c r="H84" s="8" t="s">
         <v>225</v>
       </c>
       <c r="I84" s="5" t="s">
@@ -3044,12 +3044,12 @@
       </c>
     </row>
     <row r="85" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B85" s="9"/>
-      <c r="C85" s="9"/>
-      <c r="D85" s="9"/>
-      <c r="E85" s="9"/>
-      <c r="F85" s="9"/>
-      <c r="G85" s="9"/>
+      <c r="B85" s="17"/>
+      <c r="C85" s="17"/>
+      <c r="D85" s="17"/>
+      <c r="E85" s="17"/>
+      <c r="F85" s="17"/>
+      <c r="G85" s="17"/>
       <c r="H85" s="6" t="s">
         <v>218</v>
       </c>
@@ -3058,22 +3058,22 @@
       </c>
     </row>
     <row r="86" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B86" s="11" t="s">
+      <c r="B86" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="C86" s="7" t="s">
+      <c r="C86" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D86" s="10" t="s">
+      <c r="D86" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="E86" s="10" t="s">
+      <c r="E86" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="F86" s="12" t="s">
+      <c r="F86" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="G86" s="7" t="s">
+      <c r="G86" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H86" s="5" t="s">
@@ -3084,12 +3084,12 @@
       </c>
     </row>
     <row r="87" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B87" s="8"/>
-      <c r="C87" s="8"/>
-      <c r="D87" s="8"/>
-      <c r="E87" s="8"/>
-      <c r="F87" s="8"/>
-      <c r="G87" s="8"/>
+      <c r="B87" s="16"/>
+      <c r="C87" s="16"/>
+      <c r="D87" s="16"/>
+      <c r="E87" s="16"/>
+      <c r="F87" s="16"/>
+      <c r="G87" s="16"/>
       <c r="H87" s="5" t="s">
         <v>218</v>
       </c>
@@ -3098,12 +3098,12 @@
       </c>
     </row>
     <row r="88" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B88" s="9"/>
-      <c r="C88" s="9"/>
-      <c r="D88" s="9"/>
-      <c r="E88" s="9"/>
-      <c r="F88" s="9"/>
-      <c r="G88" s="9"/>
+      <c r="B88" s="17"/>
+      <c r="C88" s="17"/>
+      <c r="D88" s="17"/>
+      <c r="E88" s="17"/>
+      <c r="F88" s="17"/>
+      <c r="G88" s="17"/>
       <c r="H88" s="6" t="s">
         <v>217</v>
       </c>
@@ -3112,22 +3112,22 @@
       </c>
     </row>
     <row r="89" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B89" s="11" t="s">
+      <c r="B89" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="C89" s="7" t="s">
+      <c r="C89" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D89" s="10" t="s">
+      <c r="D89" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="E89" s="10" t="s">
+      <c r="E89" s="20" t="s">
         <v>99</v>
       </c>
-      <c r="F89" s="12" t="s">
+      <c r="F89" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="G89" s="7" t="s">
+      <c r="G89" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H89" s="5" t="s">
@@ -3138,12 +3138,12 @@
       </c>
     </row>
     <row r="90" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B90" s="8"/>
-      <c r="C90" s="8"/>
-      <c r="D90" s="8"/>
-      <c r="E90" s="8"/>
-      <c r="F90" s="8"/>
-      <c r="G90" s="8"/>
+      <c r="B90" s="16"/>
+      <c r="C90" s="16"/>
+      <c r="D90" s="16"/>
+      <c r="E90" s="16"/>
+      <c r="F90" s="16"/>
+      <c r="G90" s="16"/>
       <c r="H90" s="5" t="s">
         <v>219</v>
       </c>
@@ -3152,12 +3152,12 @@
       </c>
     </row>
     <row r="91" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B91" s="8"/>
-      <c r="C91" s="8"/>
-      <c r="D91" s="8"/>
-      <c r="E91" s="8"/>
-      <c r="F91" s="8"/>
-      <c r="G91" s="8"/>
+      <c r="B91" s="16"/>
+      <c r="C91" s="16"/>
+      <c r="D91" s="16"/>
+      <c r="E91" s="16"/>
+      <c r="F91" s="16"/>
+      <c r="G91" s="16"/>
       <c r="H91" s="5" t="s">
         <v>225</v>
       </c>
@@ -3166,12 +3166,12 @@
       </c>
     </row>
     <row r="92" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B92" s="9"/>
-      <c r="C92" s="9"/>
-      <c r="D92" s="9"/>
-      <c r="E92" s="9"/>
-      <c r="F92" s="9"/>
-      <c r="G92" s="9"/>
+      <c r="B92" s="17"/>
+      <c r="C92" s="17"/>
+      <c r="D92" s="17"/>
+      <c r="E92" s="17"/>
+      <c r="F92" s="17"/>
+      <c r="G92" s="17"/>
       <c r="H92" s="6" t="s">
         <v>218</v>
       </c>
@@ -3180,22 +3180,22 @@
       </c>
     </row>
     <row r="93" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B93" s="11" t="s">
+      <c r="B93" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="C93" s="7" t="s">
+      <c r="C93" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D93" s="10" t="s">
+      <c r="D93" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="E93" s="10" t="s">
+      <c r="E93" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="F93" s="12" t="s">
+      <c r="F93" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="G93" s="7" t="s">
+      <c r="G93" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H93" s="5" t="s">
@@ -3206,12 +3206,12 @@
       </c>
     </row>
     <row r="94" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B94" s="8"/>
-      <c r="C94" s="8"/>
-      <c r="D94" s="8"/>
-      <c r="E94" s="8"/>
-      <c r="F94" s="8"/>
-      <c r="G94" s="8"/>
+      <c r="B94" s="16"/>
+      <c r="C94" s="16"/>
+      <c r="D94" s="16"/>
+      <c r="E94" s="16"/>
+      <c r="F94" s="16"/>
+      <c r="G94" s="16"/>
       <c r="H94" s="5" t="s">
         <v>219</v>
       </c>
@@ -3220,12 +3220,12 @@
       </c>
     </row>
     <row r="95" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B95" s="8"/>
-      <c r="C95" s="8"/>
-      <c r="D95" s="8"/>
-      <c r="E95" s="8"/>
-      <c r="F95" s="8"/>
-      <c r="G95" s="8"/>
+      <c r="B95" s="16"/>
+      <c r="C95" s="16"/>
+      <c r="D95" s="16"/>
+      <c r="E95" s="16"/>
+      <c r="F95" s="16"/>
+      <c r="G95" s="16"/>
       <c r="H95" s="5" t="s">
         <v>218</v>
       </c>
@@ -3234,12 +3234,12 @@
       </c>
     </row>
     <row r="96" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B96" s="9"/>
-      <c r="C96" s="9"/>
-      <c r="D96" s="9"/>
-      <c r="E96" s="9"/>
-      <c r="F96" s="9"/>
-      <c r="G96" s="9"/>
+      <c r="B96" s="17"/>
+      <c r="C96" s="17"/>
+      <c r="D96" s="17"/>
+      <c r="E96" s="17"/>
+      <c r="F96" s="17"/>
+      <c r="G96" s="17"/>
       <c r="H96" s="6" t="s">
         <v>212</v>
       </c>
@@ -3248,22 +3248,22 @@
       </c>
     </row>
     <row r="97" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B97" s="11" t="s">
+      <c r="B97" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="C97" s="7" t="s">
+      <c r="C97" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D97" s="10" t="s">
+      <c r="D97" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="E97" s="10" t="s">
+      <c r="E97" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="F97" s="12" t="s">
+      <c r="F97" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="G97" s="7" t="s">
+      <c r="G97" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H97" s="5" t="s">
@@ -3274,12 +3274,12 @@
       </c>
     </row>
     <row r="98" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B98" s="8"/>
-      <c r="C98" s="8"/>
-      <c r="D98" s="8"/>
-      <c r="E98" s="8"/>
-      <c r="F98" s="8"/>
-      <c r="G98" s="8"/>
+      <c r="B98" s="16"/>
+      <c r="C98" s="16"/>
+      <c r="D98" s="16"/>
+      <c r="E98" s="16"/>
+      <c r="F98" s="16"/>
+      <c r="G98" s="16"/>
       <c r="H98" s="5" t="s">
         <v>219</v>
       </c>
@@ -3288,12 +3288,12 @@
       </c>
     </row>
     <row r="99" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B99" s="8"/>
-      <c r="C99" s="8"/>
-      <c r="D99" s="8"/>
-      <c r="E99" s="8"/>
-      <c r="F99" s="8"/>
-      <c r="G99" s="8"/>
+      <c r="B99" s="16"/>
+      <c r="C99" s="16"/>
+      <c r="D99" s="16"/>
+      <c r="E99" s="16"/>
+      <c r="F99" s="16"/>
+      <c r="G99" s="16"/>
       <c r="H99" s="5" t="s">
         <v>228</v>
       </c>
@@ -3302,12 +3302,12 @@
       </c>
     </row>
     <row r="100" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B100" s="8"/>
-      <c r="C100" s="8"/>
-      <c r="D100" s="8"/>
-      <c r="E100" s="8"/>
-      <c r="F100" s="8"/>
-      <c r="G100" s="8"/>
+      <c r="B100" s="16"/>
+      <c r="C100" s="16"/>
+      <c r="D100" s="16"/>
+      <c r="E100" s="16"/>
+      <c r="F100" s="16"/>
+      <c r="G100" s="16"/>
       <c r="H100" s="5" t="s">
         <v>217</v>
       </c>
@@ -3316,12 +3316,12 @@
       </c>
     </row>
     <row r="101" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B101" s="9"/>
-      <c r="C101" s="9"/>
-      <c r="D101" s="9"/>
-      <c r="E101" s="9"/>
-      <c r="F101" s="9"/>
-      <c r="G101" s="9"/>
+      <c r="B101" s="17"/>
+      <c r="C101" s="17"/>
+      <c r="D101" s="17"/>
+      <c r="E101" s="17"/>
+      <c r="F101" s="17"/>
+      <c r="G101" s="17"/>
       <c r="H101" s="6" t="s">
         <v>229</v>
       </c>
@@ -3330,22 +3330,22 @@
       </c>
     </row>
     <row r="102" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B102" s="11" t="s">
+      <c r="B102" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="C102" s="7" t="s">
+      <c r="C102" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D102" s="10" t="s">
+      <c r="D102" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="E102" s="10" t="s">
+      <c r="E102" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="F102" s="12" t="s">
+      <c r="F102" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="G102" s="7" t="s">
+      <c r="G102" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H102" s="5" t="s">
@@ -3356,12 +3356,12 @@
       </c>
     </row>
     <row r="103" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B103" s="8"/>
-      <c r="C103" s="8"/>
-      <c r="D103" s="8"/>
-      <c r="E103" s="8"/>
-      <c r="F103" s="8"/>
-      <c r="G103" s="8"/>
+      <c r="B103" s="16"/>
+      <c r="C103" s="16"/>
+      <c r="D103" s="16"/>
+      <c r="E103" s="16"/>
+      <c r="F103" s="16"/>
+      <c r="G103" s="16"/>
       <c r="H103" s="5" t="s">
         <v>212</v>
       </c>
@@ -3370,12 +3370,12 @@
       </c>
     </row>
     <row r="104" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B104" s="8"/>
-      <c r="C104" s="8"/>
-      <c r="D104" s="8"/>
-      <c r="E104" s="8"/>
-      <c r="F104" s="8"/>
-      <c r="G104" s="8"/>
+      <c r="B104" s="16"/>
+      <c r="C104" s="16"/>
+      <c r="D104" s="16"/>
+      <c r="E104" s="16"/>
+      <c r="F104" s="16"/>
+      <c r="G104" s="16"/>
       <c r="H104" s="5" t="s">
         <v>218</v>
       </c>
@@ -3384,12 +3384,12 @@
       </c>
     </row>
     <row r="105" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B105" s="9"/>
-      <c r="C105" s="9"/>
-      <c r="D105" s="9"/>
-      <c r="E105" s="9"/>
-      <c r="F105" s="9"/>
-      <c r="G105" s="9"/>
+      <c r="B105" s="17"/>
+      <c r="C105" s="17"/>
+      <c r="D105" s="17"/>
+      <c r="E105" s="17"/>
+      <c r="F105" s="17"/>
+      <c r="G105" s="17"/>
       <c r="H105" s="6" t="s">
         <v>217</v>
       </c>
@@ -3398,22 +3398,22 @@
       </c>
     </row>
     <row r="106" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B106" s="11" t="s">
+      <c r="B106" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="C106" s="7" t="s">
+      <c r="C106" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D106" s="10" t="s">
+      <c r="D106" s="20" t="s">
         <v>114</v>
       </c>
-      <c r="E106" s="10" t="s">
+      <c r="E106" s="20" t="s">
         <v>115</v>
       </c>
-      <c r="F106" s="12" t="s">
+      <c r="F106" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="G106" s="7" t="s">
+      <c r="G106" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H106" s="5" t="s">
@@ -3424,12 +3424,12 @@
       </c>
     </row>
     <row r="107" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B107" s="8"/>
-      <c r="C107" s="8"/>
-      <c r="D107" s="8"/>
-      <c r="E107" s="8"/>
-      <c r="F107" s="8"/>
-      <c r="G107" s="8"/>
+      <c r="B107" s="16"/>
+      <c r="C107" s="16"/>
+      <c r="D107" s="16"/>
+      <c r="E107" s="16"/>
+      <c r="F107" s="16"/>
+      <c r="G107" s="16"/>
       <c r="H107" s="5" t="s">
         <v>230</v>
       </c>
@@ -3438,12 +3438,12 @@
       </c>
     </row>
     <row r="108" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B108" s="8"/>
-      <c r="C108" s="8"/>
-      <c r="D108" s="8"/>
-      <c r="E108" s="8"/>
-      <c r="F108" s="8"/>
-      <c r="G108" s="8"/>
+      <c r="B108" s="16"/>
+      <c r="C108" s="16"/>
+      <c r="D108" s="16"/>
+      <c r="E108" s="16"/>
+      <c r="F108" s="16"/>
+      <c r="G108" s="16"/>
       <c r="H108" s="5" t="s">
         <v>218</v>
       </c>
@@ -3452,12 +3452,12 @@
       </c>
     </row>
     <row r="109" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B109" s="9"/>
-      <c r="C109" s="9"/>
-      <c r="D109" s="9"/>
-      <c r="E109" s="9"/>
-      <c r="F109" s="9"/>
-      <c r="G109" s="9"/>
+      <c r="B109" s="17"/>
+      <c r="C109" s="17"/>
+      <c r="D109" s="17"/>
+      <c r="E109" s="17"/>
+      <c r="F109" s="17"/>
+      <c r="G109" s="17"/>
       <c r="H109" s="6" t="s">
         <v>212</v>
       </c>
@@ -3466,22 +3466,22 @@
       </c>
     </row>
     <row r="110" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B110" s="11" t="s">
+      <c r="B110" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="C110" s="7" t="s">
+      <c r="C110" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D110" s="10" t="s">
+      <c r="D110" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="E110" s="10" t="s">
+      <c r="E110" s="20" t="s">
         <v>119</v>
       </c>
-      <c r="F110" s="12" t="s">
+      <c r="F110" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="G110" s="7" t="s">
+      <c r="G110" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H110" s="5" t="s">
@@ -3492,12 +3492,12 @@
       </c>
     </row>
     <row r="111" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B111" s="8"/>
-      <c r="C111" s="8"/>
-      <c r="D111" s="8"/>
-      <c r="E111" s="8"/>
-      <c r="F111" s="8"/>
-      <c r="G111" s="8"/>
+      <c r="B111" s="16"/>
+      <c r="C111" s="16"/>
+      <c r="D111" s="16"/>
+      <c r="E111" s="16"/>
+      <c r="F111" s="16"/>
+      <c r="G111" s="16"/>
       <c r="H111" s="5" t="s">
         <v>210</v>
       </c>
@@ -3506,26 +3506,26 @@
       </c>
     </row>
     <row r="112" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B112" s="8"/>
-      <c r="C112" s="8"/>
-      <c r="D112" s="8"/>
-      <c r="E112" s="8"/>
-      <c r="F112" s="8"/>
-      <c r="G112" s="8"/>
-      <c r="H112" s="17" t="s">
+      <c r="B112" s="16"/>
+      <c r="C112" s="16"/>
+      <c r="D112" s="16"/>
+      <c r="E112" s="16"/>
+      <c r="F112" s="16"/>
+      <c r="G112" s="16"/>
+      <c r="H112" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="I112" s="17" t="s">
+      <c r="I112" s="10" t="s">
         <v>321</v>
       </c>
     </row>
     <row r="113" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B113" s="9"/>
-      <c r="C113" s="9"/>
-      <c r="D113" s="9"/>
-      <c r="E113" s="9"/>
-      <c r="F113" s="9"/>
-      <c r="G113" s="9"/>
+      <c r="B113" s="17"/>
+      <c r="C113" s="17"/>
+      <c r="D113" s="17"/>
+      <c r="E113" s="17"/>
+      <c r="F113" s="17"/>
+      <c r="G113" s="17"/>
       <c r="H113" s="6" t="s">
         <v>218</v>
       </c>
@@ -3534,22 +3534,22 @@
       </c>
     </row>
     <row r="114" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B114" s="11" t="s">
+      <c r="B114" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="C114" s="7" t="s">
+      <c r="C114" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D114" s="10" t="s">
+      <c r="D114" s="20" t="s">
         <v>122</v>
       </c>
-      <c r="E114" s="10" t="s">
+      <c r="E114" s="20" t="s">
         <v>123</v>
       </c>
-      <c r="F114" s="12" t="s">
+      <c r="F114" s="19" t="s">
         <v>124</v>
       </c>
-      <c r="G114" s="7" t="s">
+      <c r="G114" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H114" s="5" t="s">
@@ -3560,12 +3560,12 @@
       </c>
     </row>
     <row r="115" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B115" s="8"/>
-      <c r="C115" s="8"/>
-      <c r="D115" s="8"/>
-      <c r="E115" s="8"/>
-      <c r="F115" s="8"/>
-      <c r="G115" s="8"/>
+      <c r="B115" s="16"/>
+      <c r="C115" s="16"/>
+      <c r="D115" s="16"/>
+      <c r="E115" s="16"/>
+      <c r="F115" s="16"/>
+      <c r="G115" s="16"/>
       <c r="H115" s="5" t="s">
         <v>229</v>
       </c>
@@ -3574,12 +3574,12 @@
       </c>
     </row>
     <row r="116" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B116" s="8"/>
-      <c r="C116" s="8"/>
-      <c r="D116" s="8"/>
-      <c r="E116" s="8"/>
-      <c r="F116" s="8"/>
-      <c r="G116" s="8"/>
+      <c r="B116" s="16"/>
+      <c r="C116" s="16"/>
+      <c r="D116" s="16"/>
+      <c r="E116" s="16"/>
+      <c r="F116" s="16"/>
+      <c r="G116" s="16"/>
       <c r="H116" s="5" t="s">
         <v>218</v>
       </c>
@@ -3588,12 +3588,12 @@
       </c>
     </row>
     <row r="117" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B117" s="9"/>
-      <c r="C117" s="9"/>
-      <c r="D117" s="9"/>
-      <c r="E117" s="9"/>
-      <c r="F117" s="9"/>
-      <c r="G117" s="9"/>
+      <c r="B117" s="17"/>
+      <c r="C117" s="17"/>
+      <c r="D117" s="17"/>
+      <c r="E117" s="17"/>
+      <c r="F117" s="17"/>
+      <c r="G117" s="17"/>
       <c r="H117" s="6" t="s">
         <v>212</v>
       </c>
@@ -3602,22 +3602,22 @@
       </c>
     </row>
     <row r="118" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B118" s="11" t="s">
+      <c r="B118" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="C118" s="7" t="s">
+      <c r="C118" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D118" s="10" t="s">
+      <c r="D118" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="E118" s="10" t="s">
+      <c r="E118" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="F118" s="12" t="s">
+      <c r="F118" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="G118" s="7" t="s">
+      <c r="G118" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H118" s="5" t="s">
@@ -3628,12 +3628,12 @@
       </c>
     </row>
     <row r="119" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B119" s="8"/>
-      <c r="C119" s="8"/>
-      <c r="D119" s="8"/>
-      <c r="E119" s="8"/>
-      <c r="F119" s="8"/>
-      <c r="G119" s="8"/>
+      <c r="B119" s="16"/>
+      <c r="C119" s="16"/>
+      <c r="D119" s="16"/>
+      <c r="E119" s="16"/>
+      <c r="F119" s="16"/>
+      <c r="G119" s="16"/>
       <c r="H119" s="5" t="s">
         <v>212</v>
       </c>
@@ -3642,12 +3642,12 @@
       </c>
     </row>
     <row r="120" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B120" s="8"/>
-      <c r="C120" s="8"/>
-      <c r="D120" s="8"/>
-      <c r="E120" s="8"/>
-      <c r="F120" s="8"/>
-      <c r="G120" s="8"/>
+      <c r="B120" s="16"/>
+      <c r="C120" s="16"/>
+      <c r="D120" s="16"/>
+      <c r="E120" s="16"/>
+      <c r="F120" s="16"/>
+      <c r="G120" s="16"/>
       <c r="H120" s="5" t="s">
         <v>218</v>
       </c>
@@ -3656,32 +3656,32 @@
       </c>
     </row>
     <row r="121" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B121" s="9"/>
-      <c r="C121" s="9"/>
-      <c r="D121" s="9"/>
-      <c r="E121" s="9"/>
-      <c r="F121" s="9"/>
-      <c r="G121" s="9"/>
+      <c r="B121" s="17"/>
+      <c r="C121" s="17"/>
+      <c r="D121" s="17"/>
+      <c r="E121" s="17"/>
+      <c r="F121" s="17"/>
+      <c r="G121" s="17"/>
       <c r="H121" s="6"/>
       <c r="I121" s="6"/>
     </row>
     <row r="122" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B122" s="11" t="s">
+      <c r="B122" s="18" t="s">
         <v>129</v>
       </c>
-      <c r="C122" s="7" t="s">
+      <c r="C122" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D122" s="10" t="s">
+      <c r="D122" s="20" t="s">
         <v>130</v>
       </c>
-      <c r="E122" s="10" t="s">
+      <c r="E122" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="F122" s="12" t="s">
+      <c r="F122" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="G122" s="7" t="s">
+      <c r="G122" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H122" s="5" t="s">
@@ -3692,12 +3692,12 @@
       </c>
     </row>
     <row r="123" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B123" s="8"/>
-      <c r="C123" s="8"/>
-      <c r="D123" s="8"/>
-      <c r="E123" s="8"/>
-      <c r="F123" s="8"/>
-      <c r="G123" s="8"/>
+      <c r="B123" s="16"/>
+      <c r="C123" s="16"/>
+      <c r="D123" s="16"/>
+      <c r="E123" s="16"/>
+      <c r="F123" s="16"/>
+      <c r="G123" s="16"/>
       <c r="H123" s="5" t="s">
         <v>218</v>
       </c>
@@ -3706,12 +3706,12 @@
       </c>
     </row>
     <row r="124" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B124" s="8"/>
-      <c r="C124" s="8"/>
-      <c r="D124" s="8"/>
-      <c r="E124" s="8"/>
-      <c r="F124" s="8"/>
-      <c r="G124" s="8"/>
+      <c r="B124" s="16"/>
+      <c r="C124" s="16"/>
+      <c r="D124" s="16"/>
+      <c r="E124" s="16"/>
+      <c r="F124" s="16"/>
+      <c r="G124" s="16"/>
       <c r="H124" s="5" t="s">
         <v>212</v>
       </c>
@@ -3720,32 +3720,32 @@
       </c>
     </row>
     <row r="125" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B125" s="9"/>
-      <c r="C125" s="9"/>
-      <c r="D125" s="9"/>
-      <c r="E125" s="9"/>
-      <c r="F125" s="9"/>
-      <c r="G125" s="9"/>
+      <c r="B125" s="17"/>
+      <c r="C125" s="17"/>
+      <c r="D125" s="17"/>
+      <c r="E125" s="17"/>
+      <c r="F125" s="17"/>
+      <c r="G125" s="17"/>
       <c r="H125" s="6"/>
       <c r="I125" s="6"/>
     </row>
     <row r="126" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B126" s="11" t="s">
+      <c r="B126" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="C126" s="7" t="s">
+      <c r="C126" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D126" s="10" t="s">
+      <c r="D126" s="20" t="s">
         <v>134</v>
       </c>
-      <c r="E126" s="10" t="s">
+      <c r="E126" s="20" t="s">
         <v>135</v>
       </c>
-      <c r="F126" s="12" t="s">
+      <c r="F126" s="19" t="s">
         <v>136</v>
       </c>
-      <c r="G126" s="7" t="s">
+      <c r="G126" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H126" s="5" t="s">
@@ -3756,12 +3756,12 @@
       </c>
     </row>
     <row r="127" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B127" s="8"/>
-      <c r="C127" s="8"/>
-      <c r="D127" s="8"/>
-      <c r="E127" s="8"/>
-      <c r="F127" s="8"/>
-      <c r="G127" s="8"/>
+      <c r="B127" s="16"/>
+      <c r="C127" s="16"/>
+      <c r="D127" s="16"/>
+      <c r="E127" s="16"/>
+      <c r="F127" s="16"/>
+      <c r="G127" s="16"/>
       <c r="H127" s="5" t="s">
         <v>212</v>
       </c>
@@ -3770,12 +3770,12 @@
       </c>
     </row>
     <row r="128" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B128" s="8"/>
-      <c r="C128" s="8"/>
-      <c r="D128" s="8"/>
-      <c r="E128" s="8"/>
-      <c r="F128" s="8"/>
-      <c r="G128" s="8"/>
+      <c r="B128" s="16"/>
+      <c r="C128" s="16"/>
+      <c r="D128" s="16"/>
+      <c r="E128" s="16"/>
+      <c r="F128" s="16"/>
+      <c r="G128" s="16"/>
       <c r="H128" s="5" t="s">
         <v>218</v>
       </c>
@@ -3784,32 +3784,32 @@
       </c>
     </row>
     <row r="129" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B129" s="9"/>
-      <c r="C129" s="9"/>
-      <c r="D129" s="9"/>
-      <c r="E129" s="9"/>
-      <c r="F129" s="9"/>
-      <c r="G129" s="9"/>
+      <c r="B129" s="17"/>
+      <c r="C129" s="17"/>
+      <c r="D129" s="17"/>
+      <c r="E129" s="17"/>
+      <c r="F129" s="17"/>
+      <c r="G129" s="17"/>
       <c r="H129" s="6"/>
       <c r="I129" s="6"/>
     </row>
     <row r="130" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B130" s="11" t="s">
+      <c r="B130" s="18" t="s">
         <v>137</v>
       </c>
-      <c r="C130" s="7" t="s">
+      <c r="C130" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D130" s="10" t="s">
+      <c r="D130" s="20" t="s">
         <v>138</v>
       </c>
-      <c r="E130" s="10" t="s">
+      <c r="E130" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="F130" s="12" t="s">
+      <c r="F130" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="G130" s="7" t="s">
+      <c r="G130" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H130" s="5" t="s">
@@ -3820,12 +3820,12 @@
       </c>
     </row>
     <row r="131" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B131" s="8"/>
-      <c r="C131" s="8"/>
-      <c r="D131" s="8"/>
-      <c r="E131" s="8"/>
-      <c r="F131" s="8"/>
-      <c r="G131" s="8"/>
+      <c r="B131" s="16"/>
+      <c r="C131" s="16"/>
+      <c r="D131" s="16"/>
+      <c r="E131" s="16"/>
+      <c r="F131" s="16"/>
+      <c r="G131" s="16"/>
       <c r="H131" s="6" t="s">
         <v>217</v>
       </c>
@@ -3834,12 +3834,12 @@
       </c>
     </row>
     <row r="132" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B132" s="8"/>
-      <c r="C132" s="8"/>
-      <c r="D132" s="8"/>
-      <c r="E132" s="8"/>
-      <c r="F132" s="8"/>
-      <c r="G132" s="8"/>
+      <c r="B132" s="16"/>
+      <c r="C132" s="16"/>
+      <c r="D132" s="16"/>
+      <c r="E132" s="16"/>
+      <c r="F132" s="16"/>
+      <c r="G132" s="16"/>
       <c r="H132" s="4" t="s">
         <v>223</v>
       </c>
@@ -3848,12 +3848,12 @@
       </c>
     </row>
     <row r="133" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B133" s="9"/>
-      <c r="C133" s="9"/>
-      <c r="D133" s="9"/>
-      <c r="E133" s="9"/>
-      <c r="F133" s="9"/>
-      <c r="G133" s="9"/>
+      <c r="B133" s="17"/>
+      <c r="C133" s="17"/>
+      <c r="D133" s="17"/>
+      <c r="E133" s="17"/>
+      <c r="F133" s="17"/>
+      <c r="G133" s="17"/>
       <c r="H133" s="4" t="s">
         <v>218</v>
       </c>
@@ -3862,22 +3862,22 @@
       </c>
     </row>
     <row r="134" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B134" s="11" t="s">
+      <c r="B134" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="C134" s="7" t="s">
+      <c r="C134" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D134" s="10" t="s">
+      <c r="D134" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="E134" s="10" t="s">
+      <c r="E134" s="20" t="s">
         <v>143</v>
       </c>
-      <c r="F134" s="12" t="s">
+      <c r="F134" s="19" t="s">
         <v>144</v>
       </c>
-      <c r="G134" s="7" t="s">
+      <c r="G134" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H134" s="5" t="s">
@@ -3888,12 +3888,12 @@
       </c>
     </row>
     <row r="135" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B135" s="8"/>
-      <c r="C135" s="8"/>
-      <c r="D135" s="8"/>
-      <c r="E135" s="8"/>
-      <c r="F135" s="8"/>
-      <c r="G135" s="8"/>
+      <c r="B135" s="16"/>
+      <c r="C135" s="16"/>
+      <c r="D135" s="16"/>
+      <c r="E135" s="16"/>
+      <c r="F135" s="16"/>
+      <c r="G135" s="16"/>
       <c r="H135" s="5" t="s">
         <v>218</v>
       </c>
@@ -3902,12 +3902,12 @@
       </c>
     </row>
     <row r="136" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B136" s="8"/>
-      <c r="C136" s="8"/>
-      <c r="D136" s="8"/>
-      <c r="E136" s="8"/>
-      <c r="F136" s="8"/>
-      <c r="G136" s="8"/>
+      <c r="B136" s="16"/>
+      <c r="C136" s="16"/>
+      <c r="D136" s="16"/>
+      <c r="E136" s="16"/>
+      <c r="F136" s="16"/>
+      <c r="G136" s="16"/>
       <c r="H136" s="5" t="s">
         <v>212</v>
       </c>
@@ -3916,32 +3916,32 @@
       </c>
     </row>
     <row r="137" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B137" s="9"/>
-      <c r="C137" s="9"/>
-      <c r="D137" s="9"/>
-      <c r="E137" s="9"/>
-      <c r="F137" s="9"/>
-      <c r="G137" s="9"/>
+      <c r="B137" s="17"/>
+      <c r="C137" s="17"/>
+      <c r="D137" s="17"/>
+      <c r="E137" s="17"/>
+      <c r="F137" s="17"/>
+      <c r="G137" s="17"/>
       <c r="H137" s="6"/>
       <c r="I137" s="6"/>
     </row>
     <row r="138" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B138" s="11" t="s">
+      <c r="B138" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="C138" s="7" t="s">
+      <c r="C138" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D138" s="10" t="s">
+      <c r="D138" s="20" t="s">
         <v>146</v>
       </c>
-      <c r="E138" s="10" t="s">
+      <c r="E138" s="20" t="s">
         <v>147</v>
       </c>
-      <c r="F138" s="12" t="s">
+      <c r="F138" s="19" t="s">
         <v>148</v>
       </c>
-      <c r="G138" s="7" t="s">
+      <c r="G138" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H138" s="5" t="s">
@@ -3952,12 +3952,12 @@
       </c>
     </row>
     <row r="139" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B139" s="8"/>
-      <c r="C139" s="8"/>
-      <c r="D139" s="8"/>
-      <c r="E139" s="8"/>
-      <c r="F139" s="8"/>
-      <c r="G139" s="8"/>
+      <c r="B139" s="16"/>
+      <c r="C139" s="16"/>
+      <c r="D139" s="16"/>
+      <c r="E139" s="16"/>
+      <c r="F139" s="16"/>
+      <c r="G139" s="16"/>
       <c r="H139" s="5" t="s">
         <v>217</v>
       </c>
@@ -3966,12 +3966,12 @@
       </c>
     </row>
     <row r="140" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B140" s="8"/>
-      <c r="C140" s="8"/>
-      <c r="D140" s="8"/>
-      <c r="E140" s="8"/>
-      <c r="F140" s="8"/>
-      <c r="G140" s="8"/>
+      <c r="B140" s="16"/>
+      <c r="C140" s="16"/>
+      <c r="D140" s="16"/>
+      <c r="E140" s="16"/>
+      <c r="F140" s="16"/>
+      <c r="G140" s="16"/>
       <c r="H140" s="5" t="s">
         <v>219</v>
       </c>
@@ -3980,12 +3980,12 @@
       </c>
     </row>
     <row r="141" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B141" s="9"/>
-      <c r="C141" s="9"/>
-      <c r="D141" s="9"/>
-      <c r="E141" s="9"/>
-      <c r="F141" s="9"/>
-      <c r="G141" s="9"/>
+      <c r="B141" s="17"/>
+      <c r="C141" s="17"/>
+      <c r="D141" s="17"/>
+      <c r="E141" s="17"/>
+      <c r="F141" s="17"/>
+      <c r="G141" s="17"/>
       <c r="H141" s="6" t="s">
         <v>218</v>
       </c>
@@ -3994,22 +3994,22 @@
       </c>
     </row>
     <row r="142" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B142" s="11" t="s">
+      <c r="B142" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="C142" s="7" t="s">
+      <c r="C142" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="D142" s="10" t="s">
+      <c r="D142" s="20" t="s">
         <v>150</v>
       </c>
-      <c r="E142" s="10" t="s">
+      <c r="E142" s="20" t="s">
         <v>151</v>
       </c>
-      <c r="F142" s="12" t="s">
+      <c r="F142" s="19" t="s">
         <v>152</v>
       </c>
-      <c r="G142" s="7" t="s">
+      <c r="G142" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H142" s="5" t="s">
@@ -4020,12 +4020,12 @@
       </c>
     </row>
     <row r="143" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B143" s="8"/>
-      <c r="C143" s="8"/>
-      <c r="D143" s="8"/>
-      <c r="E143" s="8"/>
-      <c r="F143" s="8"/>
-      <c r="G143" s="8"/>
+      <c r="B143" s="16"/>
+      <c r="C143" s="16"/>
+      <c r="D143" s="16"/>
+      <c r="E143" s="16"/>
+      <c r="F143" s="16"/>
+      <c r="G143" s="16"/>
       <c r="H143" s="5" t="s">
         <v>226</v>
       </c>
@@ -4034,26 +4034,26 @@
       </c>
     </row>
     <row r="144" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B144" s="8"/>
-      <c r="C144" s="8"/>
-      <c r="D144" s="8"/>
-      <c r="E144" s="8"/>
-      <c r="F144" s="8"/>
-      <c r="G144" s="8"/>
-      <c r="H144" s="18" t="s">
+      <c r="B144" s="16"/>
+      <c r="C144" s="16"/>
+      <c r="D144" s="16"/>
+      <c r="E144" s="16"/>
+      <c r="F144" s="16"/>
+      <c r="G144" s="16"/>
+      <c r="H144" s="11" t="s">
         <v>212</v>
       </c>
-      <c r="I144" s="18" t="s">
+      <c r="I144" s="11" t="s">
         <v>344</v>
       </c>
     </row>
     <row r="145" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B145" s="9"/>
-      <c r="C145" s="9"/>
-      <c r="D145" s="9"/>
-      <c r="E145" s="9"/>
-      <c r="F145" s="9"/>
-      <c r="G145" s="9"/>
+      <c r="B145" s="17"/>
+      <c r="C145" s="17"/>
+      <c r="D145" s="17"/>
+      <c r="E145" s="17"/>
+      <c r="F145" s="17"/>
+      <c r="G145" s="17"/>
       <c r="H145" s="4" t="s">
         <v>218</v>
       </c>
@@ -4062,22 +4062,22 @@
       </c>
     </row>
     <row r="146" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B146" s="11" t="s">
+      <c r="B146" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="C146" s="7" t="s">
+      <c r="C146" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D146" s="10" t="s">
+      <c r="D146" s="20" t="s">
         <v>154</v>
       </c>
-      <c r="E146" s="10" t="s">
+      <c r="E146" s="20" t="s">
         <v>155</v>
       </c>
-      <c r="F146" s="12" t="s">
+      <c r="F146" s="19" t="s">
         <v>156</v>
       </c>
-      <c r="G146" s="7" t="s">
+      <c r="G146" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H146" s="5" t="s">
@@ -4088,12 +4088,12 @@
       </c>
     </row>
     <row r="147" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B147" s="8"/>
-      <c r="C147" s="8"/>
-      <c r="D147" s="8"/>
-      <c r="E147" s="8"/>
-      <c r="F147" s="8"/>
-      <c r="G147" s="8"/>
+      <c r="B147" s="16"/>
+      <c r="C147" s="16"/>
+      <c r="D147" s="16"/>
+      <c r="E147" s="16"/>
+      <c r="F147" s="16"/>
+      <c r="G147" s="16"/>
       <c r="H147" s="5" t="s">
         <v>229</v>
       </c>
@@ -4102,12 +4102,12 @@
       </c>
     </row>
     <row r="148" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B148" s="8"/>
-      <c r="C148" s="8"/>
-      <c r="D148" s="8"/>
-      <c r="E148" s="8"/>
-      <c r="F148" s="8"/>
-      <c r="G148" s="8"/>
+      <c r="B148" s="16"/>
+      <c r="C148" s="16"/>
+      <c r="D148" s="16"/>
+      <c r="E148" s="16"/>
+      <c r="F148" s="16"/>
+      <c r="G148" s="16"/>
       <c r="H148" s="5" t="s">
         <v>223</v>
       </c>
@@ -4116,12 +4116,12 @@
       </c>
     </row>
     <row r="149" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B149" s="9"/>
-      <c r="C149" s="9"/>
-      <c r="D149" s="9"/>
-      <c r="E149" s="9"/>
-      <c r="F149" s="9"/>
-      <c r="G149" s="9"/>
+      <c r="B149" s="17"/>
+      <c r="C149" s="17"/>
+      <c r="D149" s="17"/>
+      <c r="E149" s="17"/>
+      <c r="F149" s="17"/>
+      <c r="G149" s="17"/>
       <c r="H149" s="6" t="s">
         <v>218</v>
       </c>
@@ -4130,22 +4130,22 @@
       </c>
     </row>
     <row r="150" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B150" s="11" t="s">
+      <c r="B150" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="C150" s="7" t="s">
+      <c r="C150" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D150" s="10" t="s">
+      <c r="D150" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="E150" s="10" t="s">
+      <c r="E150" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="F150" s="12" t="s">
+      <c r="F150" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="G150" s="7" t="s">
+      <c r="G150" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H150" s="5" t="s">
@@ -4156,12 +4156,12 @@
       </c>
     </row>
     <row r="151" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B151" s="8"/>
-      <c r="C151" s="8"/>
-      <c r="D151" s="8"/>
-      <c r="E151" s="8"/>
-      <c r="F151" s="8"/>
-      <c r="G151" s="8"/>
+      <c r="B151" s="16"/>
+      <c r="C151" s="16"/>
+      <c r="D151" s="16"/>
+      <c r="E151" s="16"/>
+      <c r="F151" s="16"/>
+      <c r="G151" s="16"/>
       <c r="H151" s="5" t="s">
         <v>217</v>
       </c>
@@ -4170,12 +4170,12 @@
       </c>
     </row>
     <row r="152" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B152" s="8"/>
-      <c r="C152" s="8"/>
-      <c r="D152" s="8"/>
-      <c r="E152" s="8"/>
-      <c r="F152" s="8"/>
-      <c r="G152" s="8"/>
+      <c r="B152" s="16"/>
+      <c r="C152" s="16"/>
+      <c r="D152" s="16"/>
+      <c r="E152" s="16"/>
+      <c r="F152" s="16"/>
+      <c r="G152" s="16"/>
       <c r="H152" s="5" t="s">
         <v>210</v>
       </c>
@@ -4184,12 +4184,12 @@
       </c>
     </row>
     <row r="153" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B153" s="8"/>
-      <c r="C153" s="8"/>
-      <c r="D153" s="8"/>
-      <c r="E153" s="8"/>
-      <c r="F153" s="8"/>
-      <c r="G153" s="8"/>
+      <c r="B153" s="16"/>
+      <c r="C153" s="16"/>
+      <c r="D153" s="16"/>
+      <c r="E153" s="16"/>
+      <c r="F153" s="16"/>
+      <c r="G153" s="16"/>
       <c r="H153" s="5" t="s">
         <v>219</v>
       </c>
@@ -4198,12 +4198,12 @@
       </c>
     </row>
     <row r="154" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B154" s="9"/>
-      <c r="C154" s="9"/>
-      <c r="D154" s="9"/>
-      <c r="E154" s="9"/>
-      <c r="F154" s="9"/>
-      <c r="G154" s="9"/>
+      <c r="B154" s="17"/>
+      <c r="C154" s="17"/>
+      <c r="D154" s="17"/>
+      <c r="E154" s="17"/>
+      <c r="F154" s="17"/>
+      <c r="G154" s="17"/>
       <c r="H154" s="6" t="s">
         <v>218</v>
       </c>
@@ -4212,22 +4212,22 @@
       </c>
     </row>
     <row r="155" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B155" s="11" t="s">
+      <c r="B155" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="C155" s="7" t="s">
+      <c r="C155" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D155" s="10" t="s">
+      <c r="D155" s="20" t="s">
         <v>162</v>
       </c>
-      <c r="E155" s="10" t="s">
+      <c r="E155" s="20" t="s">
         <v>163</v>
       </c>
-      <c r="F155" s="12" t="s">
+      <c r="F155" s="19" t="s">
         <v>164</v>
       </c>
-      <c r="G155" s="7" t="s">
+      <c r="G155" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H155" s="5" t="s">
@@ -4238,12 +4238,12 @@
       </c>
     </row>
     <row r="156" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B156" s="8"/>
-      <c r="C156" s="8"/>
-      <c r="D156" s="8"/>
-      <c r="E156" s="8"/>
-      <c r="F156" s="8"/>
-      <c r="G156" s="8"/>
+      <c r="B156" s="16"/>
+      <c r="C156" s="16"/>
+      <c r="D156" s="16"/>
+      <c r="E156" s="16"/>
+      <c r="F156" s="16"/>
+      <c r="G156" s="16"/>
       <c r="H156" s="5" t="s">
         <v>217</v>
       </c>
@@ -4252,12 +4252,12 @@
       </c>
     </row>
     <row r="157" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B157" s="8"/>
-      <c r="C157" s="8"/>
-      <c r="D157" s="8"/>
-      <c r="E157" s="8"/>
-      <c r="F157" s="8"/>
-      <c r="G157" s="8"/>
+      <c r="B157" s="16"/>
+      <c r="C157" s="16"/>
+      <c r="D157" s="16"/>
+      <c r="E157" s="16"/>
+      <c r="F157" s="16"/>
+      <c r="G157" s="16"/>
       <c r="H157" s="5" t="s">
         <v>218</v>
       </c>
@@ -4266,12 +4266,12 @@
       </c>
     </row>
     <row r="158" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B158" s="9"/>
-      <c r="C158" s="9"/>
-      <c r="D158" s="9"/>
-      <c r="E158" s="9"/>
-      <c r="F158" s="9"/>
-      <c r="G158" s="9"/>
+      <c r="B158" s="17"/>
+      <c r="C158" s="17"/>
+      <c r="D158" s="17"/>
+      <c r="E158" s="17"/>
+      <c r="F158" s="17"/>
+      <c r="G158" s="17"/>
       <c r="H158" s="6" t="s">
         <v>223</v>
       </c>
@@ -4280,22 +4280,22 @@
       </c>
     </row>
     <row r="159" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B159" s="11" t="s">
+      <c r="B159" s="18" t="s">
         <v>165</v>
       </c>
-      <c r="C159" s="7" t="s">
+      <c r="C159" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D159" s="10" t="s">
+      <c r="D159" s="20" t="s">
         <v>166</v>
       </c>
-      <c r="E159" s="10" t="s">
+      <c r="E159" s="20" t="s">
         <v>167</v>
       </c>
-      <c r="F159" s="12" t="s">
+      <c r="F159" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="G159" s="7" t="s">
+      <c r="G159" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H159" s="5" t="s">
@@ -4306,12 +4306,12 @@
       </c>
     </row>
     <row r="160" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B160" s="8"/>
-      <c r="C160" s="8"/>
-      <c r="D160" s="8"/>
-      <c r="E160" s="8"/>
-      <c r="F160" s="8"/>
-      <c r="G160" s="8"/>
+      <c r="B160" s="16"/>
+      <c r="C160" s="16"/>
+      <c r="D160" s="16"/>
+      <c r="E160" s="16"/>
+      <c r="F160" s="16"/>
+      <c r="G160" s="16"/>
       <c r="H160" s="5" t="s">
         <v>224</v>
       </c>
@@ -4320,12 +4320,12 @@
       </c>
     </row>
     <row r="161" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B161" s="8"/>
-      <c r="C161" s="8"/>
-      <c r="D161" s="8"/>
-      <c r="E161" s="8"/>
-      <c r="F161" s="8"/>
-      <c r="G161" s="8"/>
+      <c r="B161" s="16"/>
+      <c r="C161" s="16"/>
+      <c r="D161" s="16"/>
+      <c r="E161" s="16"/>
+      <c r="F161" s="16"/>
+      <c r="G161" s="16"/>
       <c r="H161" s="5" t="s">
         <v>218</v>
       </c>
@@ -4334,12 +4334,12 @@
       </c>
     </row>
     <row r="162" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B162" s="9"/>
-      <c r="C162" s="9"/>
-      <c r="D162" s="9"/>
-      <c r="E162" s="9"/>
-      <c r="F162" s="9"/>
-      <c r="G162" s="9"/>
+      <c r="B162" s="17"/>
+      <c r="C162" s="17"/>
+      <c r="D162" s="17"/>
+      <c r="E162" s="17"/>
+      <c r="F162" s="17"/>
+      <c r="G162" s="17"/>
       <c r="H162" s="6" t="s">
         <v>212</v>
       </c>
@@ -4348,22 +4348,22 @@
       </c>
     </row>
     <row r="163" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B163" s="11" t="s">
+      <c r="B163" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="C163" s="7" t="s">
+      <c r="C163" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D163" s="10" t="s">
+      <c r="D163" s="20" t="s">
         <v>170</v>
       </c>
-      <c r="E163" s="10" t="s">
+      <c r="E163" s="20" t="s">
         <v>171</v>
       </c>
-      <c r="F163" s="12" t="s">
+      <c r="F163" s="19" t="s">
         <v>172</v>
       </c>
-      <c r="G163" s="7" t="s">
+      <c r="G163" s="15" t="s">
         <v>11</v>
       </c>
       <c r="H163" s="5" t="s">
@@ -4374,12 +4374,12 @@
       </c>
     </row>
     <row r="164" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B164" s="8"/>
-      <c r="C164" s="8"/>
-      <c r="D164" s="8"/>
-      <c r="E164" s="8"/>
-      <c r="F164" s="8"/>
-      <c r="G164" s="8"/>
+      <c r="B164" s="16"/>
+      <c r="C164" s="16"/>
+      <c r="D164" s="16"/>
+      <c r="E164" s="16"/>
+      <c r="F164" s="16"/>
+      <c r="G164" s="16"/>
       <c r="H164" s="5" t="s">
         <v>218</v>
       </c>
@@ -4388,12 +4388,12 @@
       </c>
     </row>
     <row r="165" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B165" s="8"/>
-      <c r="C165" s="8"/>
-      <c r="D165" s="8"/>
-      <c r="E165" s="8"/>
-      <c r="F165" s="8"/>
-      <c r="G165" s="8"/>
+      <c r="B165" s="16"/>
+      <c r="C165" s="16"/>
+      <c r="D165" s="16"/>
+      <c r="E165" s="16"/>
+      <c r="F165" s="16"/>
+      <c r="G165" s="16"/>
       <c r="H165" s="5" t="s">
         <v>212</v>
       </c>
@@ -4402,49 +4402,49 @@
       </c>
     </row>
     <row r="166" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B166" s="9"/>
-      <c r="C166" s="9"/>
-      <c r="D166" s="9"/>
-      <c r="E166" s="9"/>
-      <c r="F166" s="9"/>
-      <c r="G166" s="9"/>
+      <c r="B166" s="17"/>
+      <c r="C166" s="17"/>
+      <c r="D166" s="17"/>
+      <c r="E166" s="17"/>
+      <c r="F166" s="17"/>
+      <c r="G166" s="17"/>
       <c r="H166" s="5"/>
       <c r="I166" s="6"/>
     </row>
     <row r="167" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B167" s="11" t="s">
+      <c r="B167" s="18" t="s">
         <v>173</v>
       </c>
-      <c r="C167" s="7" t="s">
+      <c r="C167" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D167" s="10" t="s">
+      <c r="D167" s="20" t="s">
         <v>174</v>
       </c>
-      <c r="E167" s="10" t="s">
+      <c r="E167" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="F167" s="12" t="s">
+      <c r="F167" s="19" t="s">
         <v>176</v>
       </c>
-      <c r="G167" s="7" t="s">
+      <c r="G167" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="H167" s="15" t="s">
+      <c r="H167" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="I167" s="21" t="s">
+      <c r="I167" s="14" t="s">
         <v>362</v>
       </c>
     </row>
     <row r="168" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B168" s="8"/>
-      <c r="C168" s="8"/>
-      <c r="D168" s="8"/>
-      <c r="E168" s="8"/>
-      <c r="F168" s="8"/>
-      <c r="G168" s="8"/>
-      <c r="H168" s="15" t="s">
+      <c r="B168" s="16"/>
+      <c r="C168" s="16"/>
+      <c r="D168" s="16"/>
+      <c r="E168" s="16"/>
+      <c r="F168" s="16"/>
+      <c r="G168" s="16"/>
+      <c r="H168" s="8" t="s">
         <v>234</v>
       </c>
       <c r="I168" s="6" t="s">
@@ -4452,550 +4452,550 @@
       </c>
     </row>
     <row r="169" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B169" s="8"/>
-      <c r="C169" s="8"/>
-      <c r="D169" s="8"/>
-      <c r="E169" s="8"/>
-      <c r="F169" s="8"/>
-      <c r="G169" s="8"/>
-      <c r="H169" s="19" t="s">
+      <c r="B169" s="16"/>
+      <c r="C169" s="16"/>
+      <c r="D169" s="16"/>
+      <c r="E169" s="16"/>
+      <c r="F169" s="16"/>
+      <c r="G169" s="16"/>
+      <c r="H169" s="12" t="s">
         <v>218</v>
       </c>
-      <c r="I169" s="20" t="s">
+      <c r="I169" s="13" t="s">
         <v>364</v>
       </c>
     </row>
     <row r="170" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B170" s="9"/>
-      <c r="C170" s="9"/>
-      <c r="D170" s="9"/>
-      <c r="E170" s="9"/>
-      <c r="F170" s="9"/>
-      <c r="G170" s="9"/>
-      <c r="H170" s="19"/>
-      <c r="I170" s="20"/>
+      <c r="B170" s="17"/>
+      <c r="C170" s="17"/>
+      <c r="D170" s="17"/>
+      <c r="E170" s="17"/>
+      <c r="F170" s="17"/>
+      <c r="G170" s="17"/>
+      <c r="H170" s="12"/>
+      <c r="I170" s="13"/>
     </row>
     <row r="171" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B171" s="11" t="s">
+      <c r="B171" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="C171" s="7" t="s">
+      <c r="C171" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D171" s="10" t="s">
+      <c r="D171" s="20" t="s">
         <v>178</v>
       </c>
-      <c r="E171" s="10" t="s">
+      <c r="E171" s="20" t="s">
         <v>179</v>
       </c>
-      <c r="F171" s="12" t="s">
+      <c r="F171" s="19" t="s">
         <v>180</v>
       </c>
-      <c r="G171" s="7" t="s">
+      <c r="G171" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="H171" s="19" t="s">
+      <c r="H171" s="12" t="s">
         <v>210</v>
       </c>
-      <c r="I171" s="20" t="s">
+      <c r="I171" s="13" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="172" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B172" s="8"/>
-      <c r="C172" s="8"/>
-      <c r="D172" s="8"/>
-      <c r="E172" s="8"/>
-      <c r="F172" s="8"/>
-      <c r="G172" s="8"/>
-      <c r="H172" s="19" t="s">
+      <c r="B172" s="16"/>
+      <c r="C172" s="16"/>
+      <c r="D172" s="16"/>
+      <c r="E172" s="16"/>
+      <c r="F172" s="16"/>
+      <c r="G172" s="16"/>
+      <c r="H172" s="12" t="s">
         <v>236</v>
       </c>
-      <c r="I172" s="19" t="s">
+      <c r="I172" s="12" t="s">
         <v>366</v>
       </c>
     </row>
     <row r="173" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B173" s="8"/>
-      <c r="C173" s="8"/>
-      <c r="D173" s="8"/>
-      <c r="E173" s="8"/>
-      <c r="F173" s="8"/>
-      <c r="G173" s="8"/>
-      <c r="H173" s="19" t="s">
+      <c r="B173" s="16"/>
+      <c r="C173" s="16"/>
+      <c r="D173" s="16"/>
+      <c r="E173" s="16"/>
+      <c r="F173" s="16"/>
+      <c r="G173" s="16"/>
+      <c r="H173" s="12" t="s">
         <v>219</v>
       </c>
-      <c r="I173" s="19" t="s">
+      <c r="I173" s="12" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="174" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B174" s="9"/>
-      <c r="C174" s="9"/>
-      <c r="D174" s="9"/>
-      <c r="E174" s="9"/>
-      <c r="F174" s="9"/>
-      <c r="G174" s="9"/>
-      <c r="H174" s="20" t="s">
+      <c r="B174" s="17"/>
+      <c r="C174" s="17"/>
+      <c r="D174" s="17"/>
+      <c r="E174" s="17"/>
+      <c r="F174" s="17"/>
+      <c r="G174" s="17"/>
+      <c r="H174" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="I174" s="20" t="s">
+      <c r="I174" s="13" t="s">
         <v>367</v>
       </c>
     </row>
     <row r="175" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B175" s="11" t="s">
+      <c r="B175" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="C175" s="7" t="s">
+      <c r="C175" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D175" s="10" t="s">
+      <c r="D175" s="20" t="s">
         <v>182</v>
       </c>
-      <c r="E175" s="10" t="s">
+      <c r="E175" s="20" t="s">
         <v>183</v>
       </c>
-      <c r="F175" s="12" t="s">
+      <c r="F175" s="19" t="s">
         <v>184</v>
       </c>
-      <c r="G175" s="7" t="s">
+      <c r="G175" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="H175" s="20" t="s">
+      <c r="H175" s="13" t="s">
         <v>210</v>
       </c>
-      <c r="I175" s="20" t="s">
+      <c r="I175" s="13" t="s">
         <v>368</v>
       </c>
     </row>
     <row r="176" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B176" s="8"/>
-      <c r="C176" s="8"/>
-      <c r="D176" s="8"/>
-      <c r="E176" s="8"/>
-      <c r="F176" s="8"/>
-      <c r="G176" s="8"/>
-      <c r="H176" s="20" t="s">
+      <c r="B176" s="16"/>
+      <c r="C176" s="16"/>
+      <c r="D176" s="16"/>
+      <c r="E176" s="16"/>
+      <c r="F176" s="16"/>
+      <c r="G176" s="16"/>
+      <c r="H176" s="13" t="s">
         <v>216</v>
       </c>
-      <c r="I176" s="20" t="s">
+      <c r="I176" s="13" t="s">
         <v>369</v>
       </c>
     </row>
     <row r="177" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B177" s="8"/>
-      <c r="C177" s="8"/>
-      <c r="D177" s="8"/>
-      <c r="E177" s="8"/>
-      <c r="F177" s="8"/>
-      <c r="G177" s="8"/>
-      <c r="H177" s="20" t="s">
+      <c r="B177" s="16"/>
+      <c r="C177" s="16"/>
+      <c r="D177" s="16"/>
+      <c r="E177" s="16"/>
+      <c r="F177" s="16"/>
+      <c r="G177" s="16"/>
+      <c r="H177" s="13" t="s">
         <v>217</v>
       </c>
-      <c r="I177" s="20" t="s">
+      <c r="I177" s="13" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="178" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B178" s="9"/>
-      <c r="C178" s="9"/>
-      <c r="D178" s="9"/>
-      <c r="E178" s="9"/>
-      <c r="F178" s="9"/>
-      <c r="G178" s="9"/>
-      <c r="H178" s="20" t="s">
+      <c r="B178" s="17"/>
+      <c r="C178" s="17"/>
+      <c r="D178" s="17"/>
+      <c r="E178" s="17"/>
+      <c r="F178" s="17"/>
+      <c r="G178" s="17"/>
+      <c r="H178" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="I178" s="20" t="s">
+      <c r="I178" s="13" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="179" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B179" s="11" t="s">
+      <c r="B179" s="18" t="s">
         <v>185</v>
       </c>
-      <c r="C179" s="7" t="s">
+      <c r="C179" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D179" s="10" t="s">
+      <c r="D179" s="20" t="s">
         <v>186</v>
       </c>
-      <c r="E179" s="10" t="s">
+      <c r="E179" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="F179" s="12" t="s">
+      <c r="F179" s="19" t="s">
         <v>188</v>
       </c>
-      <c r="G179" s="7" t="s">
+      <c r="G179" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="H179" s="20" t="s">
+      <c r="H179" s="13" t="s">
         <v>223</v>
       </c>
-      <c r="I179" s="20" t="s">
+      <c r="I179" s="13" t="s">
         <v>327</v>
       </c>
     </row>
     <row r="180" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B180" s="8"/>
-      <c r="C180" s="8"/>
-      <c r="D180" s="8"/>
-      <c r="E180" s="8"/>
-      <c r="F180" s="8"/>
-      <c r="G180" s="8"/>
-      <c r="H180" s="20" t="s">
+      <c r="B180" s="16"/>
+      <c r="C180" s="16"/>
+      <c r="D180" s="16"/>
+      <c r="E180" s="16"/>
+      <c r="F180" s="16"/>
+      <c r="G180" s="16"/>
+      <c r="H180" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="I180" s="20" t="s">
+      <c r="I180" s="13" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="181" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B181" s="8"/>
-      <c r="C181" s="8"/>
-      <c r="D181" s="8"/>
-      <c r="E181" s="8"/>
-      <c r="F181" s="8"/>
-      <c r="G181" s="8"/>
-      <c r="H181" s="20" t="s">
+      <c r="B181" s="16"/>
+      <c r="C181" s="16"/>
+      <c r="D181" s="16"/>
+      <c r="E181" s="16"/>
+      <c r="F181" s="16"/>
+      <c r="G181" s="16"/>
+      <c r="H181" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="I181" s="20" t="s">
+      <c r="I181" s="13" t="s">
         <v>361</v>
       </c>
     </row>
     <row r="182" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B182" s="9"/>
-      <c r="C182" s="9"/>
-      <c r="D182" s="9"/>
-      <c r="E182" s="9"/>
-      <c r="F182" s="9"/>
-      <c r="G182" s="9"/>
-      <c r="H182" s="20"/>
-      <c r="I182" s="20"/>
+      <c r="B182" s="17"/>
+      <c r="C182" s="17"/>
+      <c r="D182" s="17"/>
+      <c r="E182" s="17"/>
+      <c r="F182" s="17"/>
+      <c r="G182" s="17"/>
+      <c r="H182" s="13"/>
+      <c r="I182" s="13"/>
     </row>
     <row r="183" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B183" s="11" t="s">
+      <c r="B183" s="18" t="s">
         <v>189</v>
       </c>
-      <c r="C183" s="7" t="s">
+      <c r="C183" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D183" s="10" t="s">
+      <c r="D183" s="20" t="s">
         <v>190</v>
       </c>
-      <c r="E183" s="10" t="s">
+      <c r="E183" s="20" t="s">
         <v>191</v>
       </c>
-      <c r="F183" s="12" t="s">
+      <c r="F183" s="19" t="s">
         <v>192</v>
       </c>
-      <c r="G183" s="7" t="s">
+      <c r="G183" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="H183" s="20" t="s">
+      <c r="H183" s="13" t="s">
         <v>223</v>
       </c>
-      <c r="I183" s="20" t="s">
+      <c r="I183" s="13" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="184" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B184" s="8"/>
-      <c r="C184" s="8"/>
-      <c r="D184" s="8"/>
-      <c r="E184" s="8"/>
-      <c r="F184" s="8"/>
-      <c r="G184" s="8"/>
-      <c r="H184" s="20" t="s">
+      <c r="B184" s="16"/>
+      <c r="C184" s="16"/>
+      <c r="D184" s="16"/>
+      <c r="E184" s="16"/>
+      <c r="F184" s="16"/>
+      <c r="G184" s="16"/>
+      <c r="H184" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="I184" s="20" t="s">
+      <c r="I184" s="13" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="185" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B185" s="8"/>
-      <c r="C185" s="8"/>
-      <c r="D185" s="8"/>
-      <c r="E185" s="8"/>
-      <c r="F185" s="8"/>
-      <c r="G185" s="8"/>
-      <c r="H185" s="20" t="s">
+      <c r="B185" s="16"/>
+      <c r="C185" s="16"/>
+      <c r="D185" s="16"/>
+      <c r="E185" s="16"/>
+      <c r="F185" s="16"/>
+      <c r="G185" s="16"/>
+      <c r="H185" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="I185" s="20" t="s">
+      <c r="I185" s="13" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="186" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B186" s="9"/>
-      <c r="C186" s="9"/>
-      <c r="D186" s="9"/>
-      <c r="E186" s="9"/>
-      <c r="F186" s="9"/>
-      <c r="G186" s="9"/>
-      <c r="H186" s="20"/>
-      <c r="I186" s="20"/>
+      <c r="B186" s="17"/>
+      <c r="C186" s="17"/>
+      <c r="D186" s="17"/>
+      <c r="E186" s="17"/>
+      <c r="F186" s="17"/>
+      <c r="G186" s="17"/>
+      <c r="H186" s="13"/>
+      <c r="I186" s="13"/>
     </row>
     <row r="187" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B187" s="11" t="s">
+      <c r="B187" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="C187" s="7" t="s">
+      <c r="C187" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D187" s="10" t="s">
+      <c r="D187" s="20" t="s">
         <v>194</v>
       </c>
-      <c r="E187" s="10" t="s">
+      <c r="E187" s="20" t="s">
         <v>195</v>
       </c>
-      <c r="F187" s="12" t="s">
+      <c r="F187" s="19" t="s">
         <v>196</v>
       </c>
-      <c r="G187" s="7" t="s">
+      <c r="G187" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="H187" s="20" t="s">
+      <c r="H187" s="13" t="s">
         <v>232</v>
       </c>
-      <c r="I187" s="20" t="s">
+      <c r="I187" s="13" t="s">
         <v>376</v>
       </c>
     </row>
     <row r="188" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B188" s="8"/>
-      <c r="C188" s="8"/>
-      <c r="D188" s="8"/>
-      <c r="E188" s="8"/>
-      <c r="F188" s="8"/>
-      <c r="G188" s="8"/>
-      <c r="H188" s="20" t="s">
+      <c r="B188" s="16"/>
+      <c r="C188" s="16"/>
+      <c r="D188" s="16"/>
+      <c r="E188" s="16"/>
+      <c r="F188" s="16"/>
+      <c r="G188" s="16"/>
+      <c r="H188" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="I188" s="20" t="s">
+      <c r="I188" s="13" t="s">
         <v>377</v>
       </c>
     </row>
     <row r="189" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B189" s="8"/>
-      <c r="C189" s="8"/>
-      <c r="D189" s="8"/>
-      <c r="E189" s="8"/>
-      <c r="F189" s="8"/>
-      <c r="G189" s="8"/>
-      <c r="H189" s="20" t="s">
+      <c r="B189" s="16"/>
+      <c r="C189" s="16"/>
+      <c r="D189" s="16"/>
+      <c r="E189" s="16"/>
+      <c r="F189" s="16"/>
+      <c r="G189" s="16"/>
+      <c r="H189" s="13" t="s">
         <v>223</v>
       </c>
-      <c r="I189" s="20" t="s">
+      <c r="I189" s="13" t="s">
         <v>378</v>
       </c>
     </row>
     <row r="190" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B190" s="9"/>
-      <c r="C190" s="9"/>
-      <c r="D190" s="9"/>
-      <c r="E190" s="9"/>
-      <c r="F190" s="9"/>
-      <c r="G190" s="9"/>
-      <c r="H190" s="20"/>
-      <c r="I190" s="20"/>
+      <c r="B190" s="17"/>
+      <c r="C190" s="17"/>
+      <c r="D190" s="17"/>
+      <c r="E190" s="17"/>
+      <c r="F190" s="17"/>
+      <c r="G190" s="17"/>
+      <c r="H190" s="13"/>
+      <c r="I190" s="13"/>
     </row>
     <row r="191" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B191" s="11" t="s">
+      <c r="B191" s="18" t="s">
         <v>197</v>
       </c>
-      <c r="C191" s="7" t="s">
+      <c r="C191" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D191" s="10" t="s">
+      <c r="D191" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="E191" s="10" t="s">
+      <c r="E191" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="F191" s="12" t="s">
+      <c r="F191" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="G191" s="7" t="s">
+      <c r="G191" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="H191" s="20" t="s">
+      <c r="H191" s="13" t="s">
         <v>223</v>
       </c>
-      <c r="I191" s="20" t="s">
+      <c r="I191" s="13" t="s">
         <v>379</v>
       </c>
     </row>
     <row r="192" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B192" s="8"/>
-      <c r="C192" s="8"/>
-      <c r="D192" s="8"/>
-      <c r="E192" s="8"/>
-      <c r="F192" s="8"/>
-      <c r="G192" s="8"/>
-      <c r="H192" s="20" t="s">
+      <c r="B192" s="16"/>
+      <c r="C192" s="16"/>
+      <c r="D192" s="16"/>
+      <c r="E192" s="16"/>
+      <c r="F192" s="16"/>
+      <c r="G192" s="16"/>
+      <c r="H192" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="I192" s="20" t="s">
+      <c r="I192" s="13" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="193" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B193" s="8"/>
-      <c r="C193" s="8"/>
-      <c r="D193" s="8"/>
-      <c r="E193" s="8"/>
-      <c r="F193" s="8"/>
-      <c r="G193" s="8"/>
-      <c r="H193" s="20" t="s">
+      <c r="B193" s="16"/>
+      <c r="C193" s="16"/>
+      <c r="D193" s="16"/>
+      <c r="E193" s="16"/>
+      <c r="F193" s="16"/>
+      <c r="G193" s="16"/>
+      <c r="H193" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="I193" s="20" t="s">
+      <c r="I193" s="13" t="s">
         <v>380</v>
       </c>
     </row>
     <row r="194" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B194" s="9"/>
-      <c r="C194" s="9"/>
-      <c r="D194" s="9"/>
-      <c r="E194" s="9"/>
-      <c r="F194" s="9"/>
-      <c r="G194" s="9"/>
-      <c r="H194" s="20"/>
-      <c r="I194" s="20"/>
+      <c r="B194" s="17"/>
+      <c r="C194" s="17"/>
+      <c r="D194" s="17"/>
+      <c r="E194" s="17"/>
+      <c r="F194" s="17"/>
+      <c r="G194" s="17"/>
+      <c r="H194" s="13"/>
+      <c r="I194" s="13"/>
     </row>
     <row r="195" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B195" s="11" t="s">
+      <c r="B195" s="18" t="s">
         <v>201</v>
       </c>
-      <c r="C195" s="7" t="s">
+      <c r="C195" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D195" s="10" t="s">
+      <c r="D195" s="20" t="s">
         <v>202</v>
       </c>
-      <c r="E195" s="10" t="s">
+      <c r="E195" s="20" t="s">
         <v>203</v>
       </c>
-      <c r="F195" s="12" t="s">
+      <c r="F195" s="19" t="s">
         <v>204</v>
       </c>
-      <c r="G195" s="7" t="s">
+      <c r="G195" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="H195" s="20" t="s">
+      <c r="H195" s="13" t="s">
         <v>223</v>
       </c>
-      <c r="I195" s="20" t="s">
+      <c r="I195" s="13" t="s">
         <v>381</v>
       </c>
     </row>
     <row r="196" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B196" s="8"/>
-      <c r="C196" s="8"/>
-      <c r="D196" s="8"/>
-      <c r="E196" s="8"/>
-      <c r="F196" s="8"/>
-      <c r="G196" s="8"/>
-      <c r="H196" s="20" t="s">
+      <c r="B196" s="16"/>
+      <c r="C196" s="16"/>
+      <c r="D196" s="16"/>
+      <c r="E196" s="16"/>
+      <c r="F196" s="16"/>
+      <c r="G196" s="16"/>
+      <c r="H196" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="I196" s="20" t="s">
+      <c r="I196" s="13" t="s">
         <v>382</v>
       </c>
     </row>
     <row r="197" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B197" s="8"/>
-      <c r="C197" s="8"/>
-      <c r="D197" s="8"/>
-      <c r="E197" s="8"/>
-      <c r="F197" s="8"/>
-      <c r="G197" s="8"/>
-      <c r="H197" s="20" t="s">
+      <c r="B197" s="16"/>
+      <c r="C197" s="16"/>
+      <c r="D197" s="16"/>
+      <c r="E197" s="16"/>
+      <c r="F197" s="16"/>
+      <c r="G197" s="16"/>
+      <c r="H197" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="I197" s="20" t="s">
+      <c r="I197" s="13" t="s">
         <v>383</v>
       </c>
     </row>
     <row r="198" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B198" s="9"/>
-      <c r="C198" s="9"/>
-      <c r="D198" s="9"/>
-      <c r="E198" s="9"/>
-      <c r="F198" s="9"/>
-      <c r="G198" s="9"/>
-      <c r="H198" s="20"/>
-      <c r="I198" s="20"/>
+      <c r="B198" s="17"/>
+      <c r="C198" s="17"/>
+      <c r="D198" s="17"/>
+      <c r="E198" s="17"/>
+      <c r="F198" s="17"/>
+      <c r="G198" s="17"/>
+      <c r="H198" s="13"/>
+      <c r="I198" s="13"/>
     </row>
     <row r="199" spans="2:9" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B199" s="11" t="s">
+      <c r="B199" s="18" t="s">
         <v>205</v>
       </c>
-      <c r="C199" s="7" t="s">
+      <c r="C199" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D199" s="10" t="s">
+      <c r="D199" s="20" t="s">
         <v>206</v>
       </c>
-      <c r="E199" s="10" t="s">
+      <c r="E199" s="20" t="s">
         <v>207</v>
       </c>
-      <c r="F199" s="12" t="s">
+      <c r="F199" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="G199" s="7" t="s">
+      <c r="G199" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="H199" s="20" t="s">
+      <c r="H199" s="13" t="s">
         <v>220</v>
       </c>
-      <c r="I199" s="20" t="s">
+      <c r="I199" s="13" t="s">
         <v>384</v>
       </c>
     </row>
     <row r="200" spans="2:9" ht="50.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B200" s="8"/>
-      <c r="C200" s="8"/>
-      <c r="D200" s="8"/>
-      <c r="E200" s="8"/>
-      <c r="F200" s="8"/>
-      <c r="G200" s="8"/>
-      <c r="H200" s="19" t="s">
+      <c r="B200" s="16"/>
+      <c r="C200" s="16"/>
+      <c r="D200" s="16"/>
+      <c r="E200" s="16"/>
+      <c r="F200" s="16"/>
+      <c r="G200" s="16"/>
+      <c r="H200" s="12" t="s">
         <v>224</v>
       </c>
-      <c r="I200" s="20" t="s">
+      <c r="I200" s="13" t="s">
         <v>329</v>
       </c>
     </row>
     <row r="201" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B201" s="8"/>
-      <c r="C201" s="8"/>
-      <c r="D201" s="8"/>
-      <c r="E201" s="8"/>
-      <c r="F201" s="8"/>
-      <c r="G201" s="8"/>
-      <c r="H201" s="20" t="s">
+      <c r="B201" s="16"/>
+      <c r="C201" s="16"/>
+      <c r="D201" s="16"/>
+      <c r="E201" s="16"/>
+      <c r="F201" s="16"/>
+      <c r="G201" s="16"/>
+      <c r="H201" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="I201" s="20" t="s">
+      <c r="I201" s="13" t="s">
         <v>385</v>
       </c>
     </row>
     <row r="202" spans="2:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B202" s="9"/>
-      <c r="C202" s="9"/>
-      <c r="D202" s="9"/>
-      <c r="E202" s="9"/>
-      <c r="F202" s="9"/>
-      <c r="G202" s="9"/>
-      <c r="H202" s="20" t="s">
+      <c r="B202" s="17"/>
+      <c r="C202" s="17"/>
+      <c r="D202" s="17"/>
+      <c r="E202" s="17"/>
+      <c r="F202" s="17"/>
+      <c r="G202" s="17"/>
+      <c r="H202" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="I202" s="20" t="s">
+      <c r="I202" s="13" t="s">
         <v>386</v>
       </c>
     </row>
@@ -5012,6 +5012,19 @@
     <mergeCell ref="B195:B198"/>
     <mergeCell ref="D159:D162"/>
     <mergeCell ref="G191:G194"/>
+    <mergeCell ref="B29:B32"/>
+    <mergeCell ref="C155:C158"/>
+    <mergeCell ref="B70:B73"/>
+    <mergeCell ref="B163:B166"/>
+    <mergeCell ref="B97:B101"/>
+    <mergeCell ref="D78:D81"/>
+    <mergeCell ref="D93:D96"/>
+    <mergeCell ref="F78:F81"/>
+    <mergeCell ref="F93:F96"/>
+    <mergeCell ref="B134:B137"/>
+    <mergeCell ref="C102:C105"/>
+    <mergeCell ref="D134:D137"/>
+    <mergeCell ref="C122:C125"/>
     <mergeCell ref="B199:B202"/>
     <mergeCell ref="D146:D149"/>
     <mergeCell ref="D199:D202"/>
@@ -5035,6 +5048,7 @@
     <mergeCell ref="F37:F41"/>
     <mergeCell ref="F142:F145"/>
     <mergeCell ref="E155:E158"/>
+    <mergeCell ref="B191:B194"/>
     <mergeCell ref="D7:D9"/>
     <mergeCell ref="D183:D186"/>
     <mergeCell ref="D70:D73"/>
@@ -5052,45 +5066,13 @@
     <mergeCell ref="E167:E170"/>
     <mergeCell ref="D175:D178"/>
     <mergeCell ref="F118:F121"/>
-    <mergeCell ref="B191:B194"/>
     <mergeCell ref="D42:D45"/>
     <mergeCell ref="D82:D85"/>
     <mergeCell ref="F82:F85"/>
-    <mergeCell ref="B29:B32"/>
     <mergeCell ref="F42:F45"/>
     <mergeCell ref="D29:D32"/>
-    <mergeCell ref="C155:C158"/>
-    <mergeCell ref="B70:B73"/>
-    <mergeCell ref="B163:B166"/>
     <mergeCell ref="D106:D109"/>
-    <mergeCell ref="B97:B101"/>
     <mergeCell ref="F106:F109"/>
-    <mergeCell ref="D78:D81"/>
-    <mergeCell ref="D93:D96"/>
-    <mergeCell ref="F78:F81"/>
-    <mergeCell ref="F93:F96"/>
-    <mergeCell ref="B134:B137"/>
-    <mergeCell ref="C102:C105"/>
-    <mergeCell ref="D134:D137"/>
-    <mergeCell ref="C122:C125"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="B126:B129"/>
-    <mergeCell ref="B110:B113"/>
-    <mergeCell ref="B187:B190"/>
-    <mergeCell ref="F50:F53"/>
-    <mergeCell ref="D130:D133"/>
-    <mergeCell ref="F130:F133"/>
-    <mergeCell ref="C150:C154"/>
-    <mergeCell ref="B171:B174"/>
-    <mergeCell ref="E150:E154"/>
-    <mergeCell ref="D171:D174"/>
-    <mergeCell ref="F114:F117"/>
-    <mergeCell ref="D155:D158"/>
-    <mergeCell ref="B175:B178"/>
-    <mergeCell ref="G17:G20"/>
-    <mergeCell ref="G130:G133"/>
-    <mergeCell ref="E58:E61"/>
-    <mergeCell ref="E163:E166"/>
     <mergeCell ref="G3:G6"/>
     <mergeCell ref="D102:D105"/>
     <mergeCell ref="E159:E162"/>
@@ -5111,11 +5093,34 @@
     <mergeCell ref="F10:F13"/>
     <mergeCell ref="F14:F16"/>
     <mergeCell ref="F25:F28"/>
+    <mergeCell ref="F50:F53"/>
+    <mergeCell ref="D130:D133"/>
+    <mergeCell ref="F130:F133"/>
+    <mergeCell ref="E150:E154"/>
+    <mergeCell ref="B179:B182"/>
+    <mergeCell ref="C50:C53"/>
+    <mergeCell ref="D195:D198"/>
+    <mergeCell ref="C142:C145"/>
+    <mergeCell ref="D179:D182"/>
+    <mergeCell ref="B66:B69"/>
+    <mergeCell ref="C183:C186"/>
+    <mergeCell ref="D58:D61"/>
+    <mergeCell ref="G17:G20"/>
+    <mergeCell ref="G130:G133"/>
+    <mergeCell ref="E58:E61"/>
+    <mergeCell ref="E163:E166"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="B126:B129"/>
+    <mergeCell ref="B110:B113"/>
+    <mergeCell ref="B187:B190"/>
+    <mergeCell ref="C150:C154"/>
+    <mergeCell ref="B171:B174"/>
+    <mergeCell ref="D171:D174"/>
+    <mergeCell ref="F114:F117"/>
+    <mergeCell ref="D155:D158"/>
+    <mergeCell ref="B175:B178"/>
     <mergeCell ref="C187:C190"/>
     <mergeCell ref="E187:E190"/>
-    <mergeCell ref="B37:B41"/>
-    <mergeCell ref="G25:G28"/>
-    <mergeCell ref="F46:F49"/>
     <mergeCell ref="F191:F194"/>
     <mergeCell ref="G159:G162"/>
     <mergeCell ref="C195:C198"/>
@@ -5129,12 +5134,10 @@
     <mergeCell ref="G179:G182"/>
     <mergeCell ref="E130:E133"/>
     <mergeCell ref="C78:C81"/>
-    <mergeCell ref="B179:B182"/>
-    <mergeCell ref="C50:C53"/>
-    <mergeCell ref="D195:D198"/>
-    <mergeCell ref="C142:C145"/>
-    <mergeCell ref="D179:D182"/>
-    <mergeCell ref="B66:B69"/>
+    <mergeCell ref="E183:E186"/>
+    <mergeCell ref="F171:F174"/>
+    <mergeCell ref="C175:C178"/>
+    <mergeCell ref="F179:F182"/>
     <mergeCell ref="C7:C9"/>
     <mergeCell ref="F97:F101"/>
     <mergeCell ref="B122:B125"/>
@@ -5279,10 +5282,9 @@
     <mergeCell ref="C54:C57"/>
     <mergeCell ref="C10:C13"/>
     <mergeCell ref="E10:E13"/>
-    <mergeCell ref="C183:C186"/>
-    <mergeCell ref="D58:D61"/>
-    <mergeCell ref="E183:E186"/>
-    <mergeCell ref="B138:B141"/>
+    <mergeCell ref="G171:G174"/>
+    <mergeCell ref="B21:B24"/>
+    <mergeCell ref="C25:C28"/>
     <mergeCell ref="E21:E24"/>
     <mergeCell ref="F58:F61"/>
     <mergeCell ref="D138:D141"/>
@@ -5294,13 +5296,11 @@
     <mergeCell ref="B155:B158"/>
     <mergeCell ref="D89:D92"/>
     <mergeCell ref="C110:C113"/>
-    <mergeCell ref="F171:F174"/>
     <mergeCell ref="F89:F92"/>
-    <mergeCell ref="C175:C178"/>
-    <mergeCell ref="F179:F182"/>
-    <mergeCell ref="G171:G174"/>
-    <mergeCell ref="B21:B24"/>
-    <mergeCell ref="C25:C28"/>
+    <mergeCell ref="B37:B41"/>
+    <mergeCell ref="G25:G28"/>
+    <mergeCell ref="F46:F49"/>
+    <mergeCell ref="B138:B141"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>